<commit_message>
Reprice offer to renovation level, add exterior scaffold, update schedule
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TY7ypkkVv2u59aH61n5dhS
</commit_message>
<xml_diff>
--- a/05_תוצרים/לוח_זמנים_שלונסקי_53.xlsx
+++ b/05_תוצרים/לוח_זמנים_שלונסקי_53.xlsx
@@ -521,7 +521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BO90"/>
+  <dimension ref="A1:BO92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1011,7 +1011,7 @@
       <c r="I7" s="9" t="n"/>
       <c r="J7" s="9" t="n"/>
       <c r="K7" s="11">
-        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$86,MATCH(E7,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(F7,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(G7,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(H7,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(I7,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(J7,$A$6:$A$86,0)),0))</f>
+        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$88,MATCH(E7,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(F7,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(G7,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(H7,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(I7,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(J7,$A$6:$A$88,0)),0))</f>
         <v/>
       </c>
       <c r="L7" s="11">
@@ -1063,7 +1063,7 @@
       <c r="I8" s="9" t="n"/>
       <c r="J8" s="9" t="n"/>
       <c r="K8" s="11">
-        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$86,MATCH(E8,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(F8,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(G8,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(H8,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(I8,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(J8,$A$6:$A$86,0)),0))</f>
+        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$88,MATCH(E8,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(F8,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(G8,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(H8,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(I8,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(J8,$A$6:$A$88,0)),0))</f>
         <v/>
       </c>
       <c r="L8" s="11">
@@ -1111,7 +1111,7 @@
       <c r="I9" s="9" t="n"/>
       <c r="J9" s="9" t="n"/>
       <c r="K9" s="11">
-        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$86,MATCH(E9,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(F9,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(G9,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(H9,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(I9,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(J9,$A$6:$A$86,0)),0))</f>
+        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$88,MATCH(E9,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(F9,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(G9,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(H9,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(I9,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(J9,$A$6:$A$88,0)),0))</f>
         <v/>
       </c>
       <c r="L9" s="11">
@@ -1163,7 +1163,7 @@
       <c r="I10" s="9" t="n"/>
       <c r="J10" s="9" t="n"/>
       <c r="K10" s="11">
-        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$86,MATCH(E10,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(F10,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(G10,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(H10,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(I10,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(J10,$A$6:$A$86,0)),0))</f>
+        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$88,MATCH(E10,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(F10,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(G10,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(H10,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(I10,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(J10,$A$6:$A$88,0)),0))</f>
         <v/>
       </c>
       <c r="L10" s="11">
@@ -1211,7 +1211,7 @@
       <c r="I11" s="9" t="n"/>
       <c r="J11" s="9" t="n"/>
       <c r="K11" s="11">
-        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$86,MATCH(E11,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(F11,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(G11,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(H11,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(I11,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(J11,$A$6:$A$86,0)),0))</f>
+        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$88,MATCH(E11,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(F11,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(G11,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(H11,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(I11,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(J11,$A$6:$A$88,0)),0))</f>
         <v/>
       </c>
       <c r="L11" s="11">
@@ -1259,7 +1259,7 @@
       <c r="I12" s="9" t="n"/>
       <c r="J12" s="9" t="n"/>
       <c r="K12" s="11">
-        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$86,MATCH(E12,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(F12,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(G12,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(H12,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(I12,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(J12,$A$6:$A$86,0)),0))</f>
+        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$88,MATCH(E12,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(F12,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(G12,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(H12,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(I12,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(J12,$A$6:$A$88,0)),0))</f>
         <v/>
       </c>
       <c r="L12" s="11">
@@ -1307,7 +1307,7 @@
       <c r="I13" s="9" t="n"/>
       <c r="J13" s="9" t="n"/>
       <c r="K13" s="11">
-        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$86,MATCH(E13,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(F13,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(G13,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(H13,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(I13,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(J13,$A$6:$A$86,0)),0))</f>
+        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$88,MATCH(E13,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(F13,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(G13,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(H13,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(I13,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(J13,$A$6:$A$88,0)),0))</f>
         <v/>
       </c>
       <c r="L13" s="11">
@@ -1355,7 +1355,7 @@
       <c r="I14" s="9" t="n"/>
       <c r="J14" s="9" t="n"/>
       <c r="K14" s="11">
-        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$86,MATCH(E14,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(F14,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(G14,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(H14,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(I14,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(J14,$A$6:$A$86,0)),0))</f>
+        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$88,MATCH(E14,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(F14,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(G14,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(H14,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(I14,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(J14,$A$6:$A$88,0)),0))</f>
         <v/>
       </c>
       <c r="L14" s="11">
@@ -1403,7 +1403,7 @@
       <c r="I15" s="9" t="n"/>
       <c r="J15" s="9" t="n"/>
       <c r="K15" s="11">
-        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$86,MATCH(E15,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(F15,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(G15,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(H15,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(I15,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(J15,$A$6:$A$86,0)),0))</f>
+        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$88,MATCH(E15,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(F15,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(G15,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(H15,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(I15,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(J15,$A$6:$A$88,0)),0))</f>
         <v/>
       </c>
       <c r="L15" s="11">
@@ -1524,7 +1524,7 @@
       <c r="I17" s="9" t="n"/>
       <c r="J17" s="9" t="n"/>
       <c r="K17" s="11">
-        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$86,MATCH(E17,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(F17,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(G17,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(H17,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(I17,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(J17,$A$6:$A$86,0)),0))</f>
+        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$88,MATCH(E17,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(F17,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(G17,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(H17,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(I17,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(J17,$A$6:$A$88,0)),0))</f>
         <v/>
       </c>
       <c r="L17" s="11">
@@ -1576,7 +1576,7 @@
       <c r="I18" s="9" t="n"/>
       <c r="J18" s="9" t="n"/>
       <c r="K18" s="11">
-        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$86,MATCH(E18,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(F18,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(G18,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(H18,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(I18,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(J18,$A$6:$A$86,0)),0))</f>
+        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$88,MATCH(E18,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(F18,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(G18,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(H18,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(I18,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(J18,$A$6:$A$88,0)),0))</f>
         <v/>
       </c>
       <c r="L18" s="11">
@@ -1628,7 +1628,7 @@
       <c r="I19" s="9" t="n"/>
       <c r="J19" s="9" t="n"/>
       <c r="K19" s="11">
-        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$86,MATCH(E19,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(F19,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(G19,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(H19,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(I19,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(J19,$A$6:$A$86,0)),0))</f>
+        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$88,MATCH(E19,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(F19,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(G19,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(H19,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(I19,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(J19,$A$6:$A$88,0)),0))</f>
         <v/>
       </c>
       <c r="L19" s="11">
@@ -1753,7 +1753,7 @@
       <c r="I21" s="9" t="n"/>
       <c r="J21" s="9" t="n"/>
       <c r="K21" s="11">
-        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$86,MATCH(E21,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(F21,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(G21,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(H21,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(I21,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(J21,$A$6:$A$86,0)),0))</f>
+        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$88,MATCH(E21,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(F21,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(G21,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(H21,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(I21,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(J21,$A$6:$A$88,0)),0))</f>
         <v/>
       </c>
       <c r="L21" s="11">
@@ -1805,7 +1805,7 @@
       <c r="I22" s="9" t="n"/>
       <c r="J22" s="9" t="n"/>
       <c r="K22" s="11">
-        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$86,MATCH(E22,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(F22,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(G22,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(H22,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(I22,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(J22,$A$6:$A$86,0)),0))</f>
+        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$88,MATCH(E22,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(F22,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(G22,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(H22,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(I22,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(J22,$A$6:$A$88,0)),0))</f>
         <v/>
       </c>
       <c r="L22" s="11">
@@ -1853,7 +1853,7 @@
       <c r="I23" s="9" t="n"/>
       <c r="J23" s="9" t="n"/>
       <c r="K23" s="11">
-        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$86,MATCH(E23,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(F23,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(G23,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(H23,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(I23,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(J23,$A$6:$A$86,0)),0))</f>
+        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$88,MATCH(E23,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(F23,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(G23,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(H23,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(I23,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(J23,$A$6:$A$88,0)),0))</f>
         <v/>
       </c>
       <c r="L23" s="11">
@@ -1901,7 +1901,7 @@
       <c r="I24" s="9" t="n"/>
       <c r="J24" s="9" t="n"/>
       <c r="K24" s="11">
-        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$86,MATCH(E24,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(F24,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(G24,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(H24,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(I24,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(J24,$A$6:$A$86,0)),0))</f>
+        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$88,MATCH(E24,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(F24,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(G24,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(H24,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(I24,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(J24,$A$6:$A$88,0)),0))</f>
         <v/>
       </c>
       <c r="L24" s="11">
@@ -1922,25 +1922,25 @@
     <row r="25">
       <c r="A25" s="9" t="inlineStr">
         <is>
-          <t>D050</t>
+          <t>X010</t>
         </is>
       </c>
       <c r="B25" s="10" t="inlineStr">
         <is>
-          <t>פירוק תקרות גבס, ריצופים (40 מ״ר), פנלים, חיפויים ומסגרות בטון (45 מ״א)</t>
+          <t>הקמת פיגום חיצוני (נשאר עד סיום טיח החזיתות והפרפט)</t>
         </is>
       </c>
       <c r="C25" s="10" t="inlineStr">
         <is>
-          <t>02.04, 02.05, 02.15, 02.18</t>
+          <t>01.09</t>
         </is>
       </c>
       <c r="D25" s="9" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="E25" s="9" t="inlineStr">
         <is>
-          <t>D010</t>
+          <t>S030</t>
         </is>
       </c>
       <c r="F25" s="9" t="n"/>
@@ -1949,7 +1949,7 @@
       <c r="I25" s="9" t="n"/>
       <c r="J25" s="9" t="n"/>
       <c r="K25" s="11">
-        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$86,MATCH(E25,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(F25,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(G25,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(H25,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(I25,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(J25,$A$6:$A$86,0)),0))</f>
+        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$88,MATCH(E25,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(F25,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(G25,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(H25,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(I25,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(J25,$A$6:$A$88,0)),0))</f>
         <v/>
       </c>
       <c r="L25" s="11">
@@ -1960,39 +1960,35 @@
         <f>IF(D25=0,L25,WORKDAY.INTL(L25,D25-1,$D$3))</f>
         <v/>
       </c>
-      <c r="N25" s="12" t="inlineStr">
-        <is>
-          <t>כן</t>
-        </is>
-      </c>
+      <c r="N25" s="9" t="n"/>
       <c r="O25" s="10" t="inlineStr">
         <is>
-          <t>הנחה</t>
+          <t>הנחה; נדרש לניסור המסגרות</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="9" t="inlineStr">
         <is>
-          <t>D060</t>
+          <t>D050</t>
         </is>
       </c>
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t>פירוק רעפים וארגזי רוח, מדרגות חוץ וגרנוליט (100 מ״ר)</t>
+          <t>פירוק תקרות גבס, ריצופים (40 מ״ר), פנלים וחיפויים</t>
         </is>
       </c>
       <c r="C26" s="10" t="inlineStr">
         <is>
-          <t>02.19, 02.20</t>
+          <t>02.04, 02.05, 02.18</t>
         </is>
       </c>
       <c r="D26" s="9" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E26" s="9" t="inlineStr">
         <is>
-          <t>S030</t>
+          <t>D010</t>
         </is>
       </c>
       <c r="F26" s="9" t="n"/>
@@ -2001,7 +1997,7 @@
       <c r="I26" s="9" t="n"/>
       <c r="J26" s="9" t="n"/>
       <c r="K26" s="11">
-        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$86,MATCH(E26,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(F26,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(G26,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(H26,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(I26,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(J26,$A$6:$A$86,0)),0))</f>
+        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$88,MATCH(E26,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(F26,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(G26,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(H26,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(I26,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(J26,$A$6:$A$88,0)),0))</f>
         <v/>
       </c>
       <c r="L26" s="11">
@@ -2012,7 +2008,11 @@
         <f>IF(D26=0,L26,WORKDAY.INTL(L26,D26-1,$D$3))</f>
         <v/>
       </c>
-      <c r="N26" s="9" t="n"/>
+      <c r="N26" s="12" t="inlineStr">
+        <is>
+          <t>כן</t>
+        </is>
+      </c>
       <c r="O26" s="10" t="inlineStr">
         <is>
           <t>הנחה</t>
@@ -2022,50 +2022,38 @@
     <row r="27">
       <c r="A27" s="9" t="inlineStr">
         <is>
-          <t>D065</t>
+          <t>D055</t>
         </is>
       </c>
       <c r="B27" s="10" t="inlineStr">
         <is>
-          <t>פינוי פסולת וניקיון יסודי</t>
+          <t>ניסור ופירוק מסגרות בטון דקורטיביות סביב חלונות (45 מ״א) מפיגום</t>
         </is>
       </c>
       <c r="C27" s="10" t="inlineStr">
         <is>
-          <t>02.16, 02.17</t>
+          <t>02.15</t>
         </is>
       </c>
       <c r="D27" s="9" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E27" s="9" t="inlineStr">
         <is>
-          <t>D020</t>
+          <t>X010</t>
         </is>
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
-          <t>D030</t>
-        </is>
-      </c>
-      <c r="G27" s="9" t="inlineStr">
-        <is>
-          <t>D040</t>
-        </is>
-      </c>
-      <c r="H27" s="9" t="inlineStr">
-        <is>
-          <t>D050</t>
-        </is>
-      </c>
-      <c r="I27" s="9" t="inlineStr">
-        <is>
-          <t>D060</t>
-        </is>
-      </c>
+          <t>D010</t>
+        </is>
+      </c>
+      <c r="G27" s="9" t="n"/>
+      <c r="H27" s="9" t="n"/>
+      <c r="I27" s="9" t="n"/>
       <c r="J27" s="9" t="n"/>
       <c r="K27" s="11">
-        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$86,MATCH(E27,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(F27,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(G27,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(H27,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(I27,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(J27,$A$6:$A$86,0)),0))</f>
+        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$88,MATCH(E27,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(F27,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(G27,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(H27,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(I27,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(J27,$A$6:$A$88,0)),0))</f>
         <v/>
       </c>
       <c r="L27" s="11">
@@ -2076,39 +2064,35 @@
         <f>IF(D27=0,L27,WORKDAY.INTL(L27,D27-1,$D$3))</f>
         <v/>
       </c>
-      <c r="N27" s="12" t="inlineStr">
-        <is>
-          <t>כן</t>
-        </is>
-      </c>
+      <c r="N27" s="9" t="n"/>
       <c r="O27" s="10" t="inlineStr">
         <is>
-          <t>הנחה</t>
+          <t>הנחה: ~9 מ״א ליום; באישור קונסטרוקטור</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="9" t="inlineStr">
         <is>
-          <t>D070</t>
+          <t>D060</t>
         </is>
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>אישור קונסטרוקטור ומתכננת למעבר לבנייה</t>
+          <t>פירוק רעפים וארגזי רוח, מדרגות חוץ וגרנוליט (100 מ״ר)</t>
         </is>
       </c>
       <c r="C28" s="10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>02.19, 02.20</t>
         </is>
       </c>
       <c r="D28" s="9" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="E28" s="9" t="inlineStr">
         <is>
-          <t>D065</t>
+          <t>S030</t>
         </is>
       </c>
       <c r="F28" s="9" t="n"/>
@@ -2117,7 +2101,7 @@
       <c r="I28" s="9" t="n"/>
       <c r="J28" s="9" t="n"/>
       <c r="K28" s="11">
-        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$86,MATCH(E28,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(F28,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(G28,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(H28,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(I28,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(J28,$A$6:$A$86,0)),0))</f>
+        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$88,MATCH(E28,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(F28,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(G28,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(H28,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(I28,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(J28,$A$6:$A$88,0)),0))</f>
         <v/>
       </c>
       <c r="L28" s="11">
@@ -2128,112 +2112,107 @@
         <f>IF(D28=0,L28,WORKDAY.INTL(L28,D28-1,$D$3))</f>
         <v/>
       </c>
-      <c r="N28" s="12" t="inlineStr">
+      <c r="N28" s="9" t="n"/>
+      <c r="O28" s="10" t="inlineStr">
+        <is>
+          <t>הנחה</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="9" t="inlineStr">
+        <is>
+          <t>D065</t>
+        </is>
+      </c>
+      <c r="B29" s="10" t="inlineStr">
+        <is>
+          <t>פינוי פסולת וניקיון יסודי</t>
+        </is>
+      </c>
+      <c r="C29" s="10" t="inlineStr">
+        <is>
+          <t>02.16, 02.17</t>
+        </is>
+      </c>
+      <c r="D29" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="E29" s="9" t="inlineStr">
+        <is>
+          <t>D020</t>
+        </is>
+      </c>
+      <c r="F29" s="9" t="inlineStr">
+        <is>
+          <t>D030</t>
+        </is>
+      </c>
+      <c r="G29" s="9" t="inlineStr">
+        <is>
+          <t>D040</t>
+        </is>
+      </c>
+      <c r="H29" s="9" t="inlineStr">
+        <is>
+          <t>D050</t>
+        </is>
+      </c>
+      <c r="I29" s="9" t="inlineStr">
+        <is>
+          <t>D055</t>
+        </is>
+      </c>
+      <c r="J29" s="9" t="inlineStr">
+        <is>
+          <t>D060</t>
+        </is>
+      </c>
+      <c r="K29" s="11">
+        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$88,MATCH(E29,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(F29,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(G29,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(H29,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(I29,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(J29,$A$6:$A$88,0)),0))</f>
+        <v/>
+      </c>
+      <c r="L29" s="11">
+        <f>IF(D29=0,IF(COUNTA(E29:J29)=0,$D$2,K29),WORKDAY.INTL(K29,1,$D$3))</f>
+        <v/>
+      </c>
+      <c r="M29" s="11">
+        <f>IF(D29=0,L29,WORKDAY.INTL(L29,D29-1,$D$3))</f>
+        <v/>
+      </c>
+      <c r="N29" s="12" t="inlineStr">
         <is>
           <t>כן</t>
         </is>
       </c>
-      <c r="O28" s="10" t="inlineStr">
-        <is>
-          <t>מפרט פרק 2</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="7" t="inlineStr">
-        <is>
-          <t>3. שלד ותוספות מבניות (לפי קונסטרוקטור)</t>
-        </is>
-      </c>
-      <c r="B29" s="8" t="n"/>
-      <c r="C29" s="8" t="n"/>
-      <c r="D29" s="8" t="n"/>
-      <c r="E29" s="8" t="n"/>
-      <c r="F29" s="8" t="n"/>
-      <c r="G29" s="8" t="n"/>
-      <c r="H29" s="8" t="n"/>
-      <c r="I29" s="8" t="n"/>
-      <c r="J29" s="8" t="n"/>
-      <c r="K29" s="8" t="n"/>
-      <c r="L29" s="8" t="n"/>
-      <c r="M29" s="8" t="n"/>
-      <c r="N29" s="8" t="n"/>
-      <c r="O29" s="8" t="n"/>
-      <c r="P29" s="8" t="n"/>
-      <c r="Q29" s="8" t="n"/>
-      <c r="R29" s="8" t="n"/>
-      <c r="S29" s="8" t="n"/>
-      <c r="T29" s="8" t="n"/>
-      <c r="U29" s="8" t="n"/>
-      <c r="V29" s="8" t="n"/>
-      <c r="W29" s="8" t="n"/>
-      <c r="X29" s="8" t="n"/>
-      <c r="Y29" s="8" t="n"/>
-      <c r="Z29" s="8" t="n"/>
-      <c r="AA29" s="8" t="n"/>
-      <c r="AB29" s="8" t="n"/>
-      <c r="AC29" s="8" t="n"/>
-      <c r="AD29" s="8" t="n"/>
-      <c r="AE29" s="8" t="n"/>
-      <c r="AF29" s="8" t="n"/>
-      <c r="AG29" s="8" t="n"/>
-      <c r="AH29" s="8" t="n"/>
-      <c r="AI29" s="8" t="n"/>
-      <c r="AJ29" s="8" t="n"/>
-      <c r="AK29" s="8" t="n"/>
-      <c r="AL29" s="8" t="n"/>
-      <c r="AM29" s="8" t="n"/>
-      <c r="AN29" s="8" t="n"/>
-      <c r="AO29" s="8" t="n"/>
-      <c r="AP29" s="8" t="n"/>
-      <c r="AQ29" s="8" t="n"/>
-      <c r="AR29" s="8" t="n"/>
-      <c r="AS29" s="8" t="n"/>
-      <c r="AT29" s="8" t="n"/>
-      <c r="AU29" s="8" t="n"/>
-      <c r="AV29" s="8" t="n"/>
-      <c r="AW29" s="8" t="n"/>
-      <c r="AX29" s="8" t="n"/>
-      <c r="AY29" s="8" t="n"/>
-      <c r="AZ29" s="8" t="n"/>
-      <c r="BA29" s="8" t="n"/>
-      <c r="BB29" s="8" t="n"/>
-      <c r="BC29" s="8" t="n"/>
-      <c r="BD29" s="8" t="n"/>
-      <c r="BE29" s="8" t="n"/>
-      <c r="BF29" s="8" t="n"/>
-      <c r="BG29" s="8" t="n"/>
-      <c r="BH29" s="8" t="n"/>
-      <c r="BI29" s="8" t="n"/>
-      <c r="BJ29" s="8" t="n"/>
-      <c r="BK29" s="8" t="n"/>
-      <c r="BL29" s="8" t="n"/>
-      <c r="BM29" s="8" t="n"/>
-      <c r="BN29" s="8" t="n"/>
-      <c r="BO29" s="8" t="n"/>
+      <c r="O29" s="10" t="inlineStr">
+        <is>
+          <t>הנחה</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="9" t="inlineStr">
         <is>
-          <t>K010</t>
+          <t>D070</t>
         </is>
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>חיזוק גרם המדרגות הפנימי</t>
+          <t>אישור קונסטרוקטור ומתכננת למעבר לבנייה</t>
         </is>
       </c>
       <c r="C30" s="10" t="inlineStr">
         <is>
-          <t>03.04</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D30" s="9" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="E30" s="9" t="inlineStr">
         <is>
-          <t>D070</t>
+          <t>D065</t>
         </is>
       </c>
       <c r="F30" s="9" t="n"/>
@@ -2242,7 +2221,7 @@
       <c r="I30" s="9" t="n"/>
       <c r="J30" s="9" t="n"/>
       <c r="K30" s="11">
-        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$86,MATCH(E30,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(F30,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(G30,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(H30,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(I30,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(J30,$A$6:$A$86,0)),0))</f>
+        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$88,MATCH(E30,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(F30,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(G30,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(H30,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(I30,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(J30,$A$6:$A$88,0)),0))</f>
         <v/>
       </c>
       <c r="L30" s="11">
@@ -2253,79 +2232,108 @@
         <f>IF(D30=0,L30,WORKDAY.INTL(L30,D30-1,$D$3))</f>
         <v/>
       </c>
-      <c r="N30" s="9" t="n"/>
+      <c r="N30" s="12" t="inlineStr">
+        <is>
+          <t>כן</t>
+        </is>
+      </c>
       <c r="O30" s="10" t="inlineStr">
         <is>
-          <t>הנחה</t>
+          <t>מפרט פרק 2</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="9" t="inlineStr">
-        <is>
-          <t>K020</t>
-        </is>
-      </c>
-      <c r="B31" s="10" t="inlineStr">
-        <is>
-          <t>כניסה חדשה וגרם מדרגות חדש</t>
-        </is>
-      </c>
-      <c r="C31" s="10" t="inlineStr">
-        <is>
-          <t>03.03</t>
-        </is>
-      </c>
-      <c r="D31" s="9" t="n">
-        <v>15</v>
-      </c>
-      <c r="E31" s="9" t="inlineStr">
-        <is>
-          <t>D070</t>
-        </is>
-      </c>
-      <c r="F31" s="9" t="n"/>
-      <c r="G31" s="9" t="n"/>
-      <c r="H31" s="9" t="n"/>
-      <c r="I31" s="9" t="n"/>
-      <c r="J31" s="9" t="n"/>
-      <c r="K31" s="11">
-        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$86,MATCH(E31,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(F31,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(G31,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(H31,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(I31,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(J31,$A$6:$A$86,0)),0))</f>
-        <v/>
-      </c>
-      <c r="L31" s="11">
-        <f>IF(D31=0,IF(COUNTA(E31:J31)=0,$D$2,K31),WORKDAY.INTL(K31,1,$D$3))</f>
-        <v/>
-      </c>
-      <c r="M31" s="11">
-        <f>IF(D31=0,L31,WORKDAY.INTL(L31,D31-1,$D$3))</f>
-        <v/>
-      </c>
-      <c r="N31" s="9" t="n"/>
-      <c r="O31" s="10" t="inlineStr">
-        <is>
-          <t>הנחה</t>
-        </is>
-      </c>
+      <c r="A31" s="7" t="inlineStr">
+        <is>
+          <t>3. שלד ותוספות מבניות (לפי קונסטרוקטור)</t>
+        </is>
+      </c>
+      <c r="B31" s="8" t="n"/>
+      <c r="C31" s="8" t="n"/>
+      <c r="D31" s="8" t="n"/>
+      <c r="E31" s="8" t="n"/>
+      <c r="F31" s="8" t="n"/>
+      <c r="G31" s="8" t="n"/>
+      <c r="H31" s="8" t="n"/>
+      <c r="I31" s="8" t="n"/>
+      <c r="J31" s="8" t="n"/>
+      <c r="K31" s="8" t="n"/>
+      <c r="L31" s="8" t="n"/>
+      <c r="M31" s="8" t="n"/>
+      <c r="N31" s="8" t="n"/>
+      <c r="O31" s="8" t="n"/>
+      <c r="P31" s="8" t="n"/>
+      <c r="Q31" s="8" t="n"/>
+      <c r="R31" s="8" t="n"/>
+      <c r="S31" s="8" t="n"/>
+      <c r="T31" s="8" t="n"/>
+      <c r="U31" s="8" t="n"/>
+      <c r="V31" s="8" t="n"/>
+      <c r="W31" s="8" t="n"/>
+      <c r="X31" s="8" t="n"/>
+      <c r="Y31" s="8" t="n"/>
+      <c r="Z31" s="8" t="n"/>
+      <c r="AA31" s="8" t="n"/>
+      <c r="AB31" s="8" t="n"/>
+      <c r="AC31" s="8" t="n"/>
+      <c r="AD31" s="8" t="n"/>
+      <c r="AE31" s="8" t="n"/>
+      <c r="AF31" s="8" t="n"/>
+      <c r="AG31" s="8" t="n"/>
+      <c r="AH31" s="8" t="n"/>
+      <c r="AI31" s="8" t="n"/>
+      <c r="AJ31" s="8" t="n"/>
+      <c r="AK31" s="8" t="n"/>
+      <c r="AL31" s="8" t="n"/>
+      <c r="AM31" s="8" t="n"/>
+      <c r="AN31" s="8" t="n"/>
+      <c r="AO31" s="8" t="n"/>
+      <c r="AP31" s="8" t="n"/>
+      <c r="AQ31" s="8" t="n"/>
+      <c r="AR31" s="8" t="n"/>
+      <c r="AS31" s="8" t="n"/>
+      <c r="AT31" s="8" t="n"/>
+      <c r="AU31" s="8" t="n"/>
+      <c r="AV31" s="8" t="n"/>
+      <c r="AW31" s="8" t="n"/>
+      <c r="AX31" s="8" t="n"/>
+      <c r="AY31" s="8" t="n"/>
+      <c r="AZ31" s="8" t="n"/>
+      <c r="BA31" s="8" t="n"/>
+      <c r="BB31" s="8" t="n"/>
+      <c r="BC31" s="8" t="n"/>
+      <c r="BD31" s="8" t="n"/>
+      <c r="BE31" s="8" t="n"/>
+      <c r="BF31" s="8" t="n"/>
+      <c r="BG31" s="8" t="n"/>
+      <c r="BH31" s="8" t="n"/>
+      <c r="BI31" s="8" t="n"/>
+      <c r="BJ31" s="8" t="n"/>
+      <c r="BK31" s="8" t="n"/>
+      <c r="BL31" s="8" t="n"/>
+      <c r="BM31" s="8" t="n"/>
+      <c r="BN31" s="8" t="n"/>
+      <c r="BO31" s="8" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="9" t="inlineStr">
         <is>
-          <t>K030</t>
+          <t>K010</t>
         </is>
       </c>
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t>הגדלת מרפסת הסלון ותוספת פרגולה</t>
+          <t>חיזוק גרם המדרגות הפנימי</t>
         </is>
       </c>
       <c r="C32" s="10" t="inlineStr">
         <is>
-          <t>03.01</t>
+          <t>03.04</t>
         </is>
       </c>
       <c r="D32" s="9" t="n">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="E32" s="9" t="inlineStr">
         <is>
@@ -2338,7 +2346,7 @@
       <c r="I32" s="9" t="n"/>
       <c r="J32" s="9" t="n"/>
       <c r="K32" s="11">
-        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$86,MATCH(E32,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(F32,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(G32,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(H32,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(I32,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(J32,$A$6:$A$86,0)),0))</f>
+        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$88,MATCH(E32,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(F32,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(G32,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(H32,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(I32,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(J32,$A$6:$A$88,0)),0))</f>
         <v/>
       </c>
       <c r="L32" s="11">
@@ -2359,21 +2367,21 @@
     <row r="33">
       <c r="A33" s="9" t="inlineStr">
         <is>
-          <t>K040</t>
+          <t>K020</t>
         </is>
       </c>
       <c r="B33" s="10" t="inlineStr">
         <is>
-          <t>תוספת חדר בקומת הגלריה</t>
+          <t>כניסה חדשה וגרם מדרגות חדש</t>
         </is>
       </c>
       <c r="C33" s="10" t="inlineStr">
         <is>
-          <t>03.02</t>
+          <t>03.03</t>
         </is>
       </c>
       <c r="D33" s="9" t="n">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="E33" s="9" t="inlineStr">
         <is>
@@ -2386,7 +2394,7 @@
       <c r="I33" s="9" t="n"/>
       <c r="J33" s="9" t="n"/>
       <c r="K33" s="11">
-        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$86,MATCH(E33,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(F33,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(G33,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(H33,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(I33,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(J33,$A$6:$A$86,0)),0))</f>
+        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$88,MATCH(E33,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(F33,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(G33,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(H33,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(I33,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(J33,$A$6:$A$88,0)),0))</f>
         <v/>
       </c>
       <c r="L33" s="11">
@@ -2397,60 +2405,44 @@
         <f>IF(D33=0,L33,WORKDAY.INTL(L33,D33-1,$D$3))</f>
         <v/>
       </c>
-      <c r="N33" s="12" t="inlineStr">
-        <is>
-          <t>כן</t>
-        </is>
-      </c>
+      <c r="N33" s="9" t="n"/>
       <c r="O33" s="10" t="inlineStr">
         <is>
-          <t>הנחה: כולל התקשות בטון</t>
+          <t>הנחה</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="9" t="inlineStr">
         <is>
-          <t>K050</t>
+          <t>K030</t>
         </is>
       </c>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>אישור קונסטרוקטור: השלד הושלם</t>
+          <t>הגדלת מרפסת הסלון ותוספת פרגולה</t>
         </is>
       </c>
       <c r="C34" s="10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>03.01</t>
         </is>
       </c>
       <c r="D34" s="9" t="n">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="E34" s="9" t="inlineStr">
         <is>
-          <t>K010</t>
-        </is>
-      </c>
-      <c r="F34" s="9" t="inlineStr">
-        <is>
-          <t>K020</t>
-        </is>
-      </c>
-      <c r="G34" s="9" t="inlineStr">
-        <is>
-          <t>K030</t>
-        </is>
-      </c>
-      <c r="H34" s="9" t="inlineStr">
-        <is>
-          <t>K040</t>
-        </is>
-      </c>
+          <t>D070</t>
+        </is>
+      </c>
+      <c r="F34" s="9" t="n"/>
+      <c r="G34" s="9" t="n"/>
+      <c r="H34" s="9" t="n"/>
       <c r="I34" s="9" t="n"/>
       <c r="J34" s="9" t="n"/>
       <c r="K34" s="11">
-        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$86,MATCH(E34,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(F34,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(G34,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(H34,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(I34,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(J34,$A$6:$A$86,0)),0))</f>
+        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$88,MATCH(E34,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(F34,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(G34,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(H34,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(I34,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(J34,$A$6:$A$88,0)),0))</f>
         <v/>
       </c>
       <c r="L34" s="11">
@@ -2461,121 +2453,108 @@
         <f>IF(D34=0,L34,WORKDAY.INTL(L34,D34-1,$D$3))</f>
         <v/>
       </c>
-      <c r="N34" s="12" t="inlineStr">
+      <c r="N34" s="9" t="n"/>
+      <c r="O34" s="10" t="inlineStr">
+        <is>
+          <t>הנחה</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="9" t="inlineStr">
+        <is>
+          <t>K040</t>
+        </is>
+      </c>
+      <c r="B35" s="10" t="inlineStr">
+        <is>
+          <t>תוספת חדר בקומת הגלריה</t>
+        </is>
+      </c>
+      <c r="C35" s="10" t="inlineStr">
+        <is>
+          <t>03.02</t>
+        </is>
+      </c>
+      <c r="D35" s="9" t="n">
+        <v>35</v>
+      </c>
+      <c r="E35" s="9" t="inlineStr">
+        <is>
+          <t>D070</t>
+        </is>
+      </c>
+      <c r="F35" s="9" t="n"/>
+      <c r="G35" s="9" t="n"/>
+      <c r="H35" s="9" t="n"/>
+      <c r="I35" s="9" t="n"/>
+      <c r="J35" s="9" t="n"/>
+      <c r="K35" s="11">
+        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$88,MATCH(E35,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(F35,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(G35,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(H35,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(I35,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(J35,$A$6:$A$88,0)),0))</f>
+        <v/>
+      </c>
+      <c r="L35" s="11">
+        <f>IF(D35=0,IF(COUNTA(E35:J35)=0,$D$2,K35),WORKDAY.INTL(K35,1,$D$3))</f>
+        <v/>
+      </c>
+      <c r="M35" s="11">
+        <f>IF(D35=0,L35,WORKDAY.INTL(L35,D35-1,$D$3))</f>
+        <v/>
+      </c>
+      <c r="N35" s="12" t="inlineStr">
         <is>
           <t>כן</t>
         </is>
       </c>
-      <c r="O34" s="10" t="inlineStr">
-        <is>
-          <t>מפרט פרק 3</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="7" t="inlineStr">
-        <is>
-          <t>4. גג ופרפט</t>
-        </is>
-      </c>
-      <c r="B35" s="8" t="n"/>
-      <c r="C35" s="8" t="n"/>
-      <c r="D35" s="8" t="n"/>
-      <c r="E35" s="8" t="n"/>
-      <c r="F35" s="8" t="n"/>
-      <c r="G35" s="8" t="n"/>
-      <c r="H35" s="8" t="n"/>
-      <c r="I35" s="8" t="n"/>
-      <c r="J35" s="8" t="n"/>
-      <c r="K35" s="8" t="n"/>
-      <c r="L35" s="8" t="n"/>
-      <c r="M35" s="8" t="n"/>
-      <c r="N35" s="8" t="n"/>
-      <c r="O35" s="8" t="n"/>
-      <c r="P35" s="8" t="n"/>
-      <c r="Q35" s="8" t="n"/>
-      <c r="R35" s="8" t="n"/>
-      <c r="S35" s="8" t="n"/>
-      <c r="T35" s="8" t="n"/>
-      <c r="U35" s="8" t="n"/>
-      <c r="V35" s="8" t="n"/>
-      <c r="W35" s="8" t="n"/>
-      <c r="X35" s="8" t="n"/>
-      <c r="Y35" s="8" t="n"/>
-      <c r="Z35" s="8" t="n"/>
-      <c r="AA35" s="8" t="n"/>
-      <c r="AB35" s="8" t="n"/>
-      <c r="AC35" s="8" t="n"/>
-      <c r="AD35" s="8" t="n"/>
-      <c r="AE35" s="8" t="n"/>
-      <c r="AF35" s="8" t="n"/>
-      <c r="AG35" s="8" t="n"/>
-      <c r="AH35" s="8" t="n"/>
-      <c r="AI35" s="8" t="n"/>
-      <c r="AJ35" s="8" t="n"/>
-      <c r="AK35" s="8" t="n"/>
-      <c r="AL35" s="8" t="n"/>
-      <c r="AM35" s="8" t="n"/>
-      <c r="AN35" s="8" t="n"/>
-      <c r="AO35" s="8" t="n"/>
-      <c r="AP35" s="8" t="n"/>
-      <c r="AQ35" s="8" t="n"/>
-      <c r="AR35" s="8" t="n"/>
-      <c r="AS35" s="8" t="n"/>
-      <c r="AT35" s="8" t="n"/>
-      <c r="AU35" s="8" t="n"/>
-      <c r="AV35" s="8" t="n"/>
-      <c r="AW35" s="8" t="n"/>
-      <c r="AX35" s="8" t="n"/>
-      <c r="AY35" s="8" t="n"/>
-      <c r="AZ35" s="8" t="n"/>
-      <c r="BA35" s="8" t="n"/>
-      <c r="BB35" s="8" t="n"/>
-      <c r="BC35" s="8" t="n"/>
-      <c r="BD35" s="8" t="n"/>
-      <c r="BE35" s="8" t="n"/>
-      <c r="BF35" s="8" t="n"/>
-      <c r="BG35" s="8" t="n"/>
-      <c r="BH35" s="8" t="n"/>
-      <c r="BI35" s="8" t="n"/>
-      <c r="BJ35" s="8" t="n"/>
-      <c r="BK35" s="8" t="n"/>
-      <c r="BL35" s="8" t="n"/>
-      <c r="BM35" s="8" t="n"/>
-      <c r="BN35" s="8" t="n"/>
-      <c r="BO35" s="8" t="n"/>
+      <c r="O35" s="10" t="inlineStr">
+        <is>
+          <t>הנחה: כולל התקשות בטון</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="9" t="inlineStr">
         <is>
-          <t>R010</t>
+          <t>K050</t>
         </is>
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>בניית פרפט חדש בהיקף הגג</t>
+          <t>אישור קונסטרוקטור: השלד הושלם</t>
         </is>
       </c>
       <c r="C36" s="10" t="inlineStr">
         <is>
-          <t>11.02</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D36" s="9" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="E36" s="9" t="inlineStr">
         <is>
-          <t>D070</t>
-        </is>
-      </c>
-      <c r="F36" s="9" t="n"/>
-      <c r="G36" s="9" t="n"/>
-      <c r="H36" s="9" t="n"/>
+          <t>K010</t>
+        </is>
+      </c>
+      <c r="F36" s="9" t="inlineStr">
+        <is>
+          <t>K020</t>
+        </is>
+      </c>
+      <c r="G36" s="9" t="inlineStr">
+        <is>
+          <t>K030</t>
+        </is>
+      </c>
+      <c r="H36" s="9" t="inlineStr">
+        <is>
+          <t>K040</t>
+        </is>
+      </c>
       <c r="I36" s="9" t="n"/>
       <c r="J36" s="9" t="n"/>
       <c r="K36" s="11">
-        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$86,MATCH(E36,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(F36,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(G36,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(H36,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(I36,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(J36,$A$6:$A$86,0)),0))</f>
+        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$88,MATCH(E36,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(F36,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(G36,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(H36,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(I36,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(J36,$A$6:$A$88,0)),0))</f>
         <v/>
       </c>
       <c r="L36" s="11">
@@ -2586,83 +2565,112 @@
         <f>IF(D36=0,L36,WORKDAY.INTL(L36,D36-1,$D$3))</f>
         <v/>
       </c>
-      <c r="N36" s="9" t="n"/>
+      <c r="N36" s="12" t="inlineStr">
+        <is>
+          <t>כן</t>
+        </is>
+      </c>
       <c r="O36" s="10" t="inlineStr">
         <is>
-          <t>הנחה; כמות לפי מדידה</t>
+          <t>מפרט פרק 3</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="9" t="inlineStr">
-        <is>
-          <t>R020</t>
-        </is>
-      </c>
-      <c r="B37" s="10" t="inlineStr">
-        <is>
-          <t>איטום גג ופרפט</t>
-        </is>
-      </c>
-      <c r="C37" s="10" t="inlineStr">
-        <is>
-          <t>11.03</t>
-        </is>
-      </c>
-      <c r="D37" s="9" t="n">
-        <v>8</v>
-      </c>
-      <c r="E37" s="9" t="inlineStr">
-        <is>
-          <t>R010</t>
-        </is>
-      </c>
-      <c r="F37" s="9" t="n"/>
-      <c r="G37" s="9" t="n"/>
-      <c r="H37" s="9" t="n"/>
-      <c r="I37" s="9" t="n"/>
-      <c r="J37" s="9" t="n"/>
-      <c r="K37" s="11">
-        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$86,MATCH(E37,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(F37,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(G37,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(H37,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(I37,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(J37,$A$6:$A$86,0)),0))</f>
-        <v/>
-      </c>
-      <c r="L37" s="11">
-        <f>IF(D37=0,IF(COUNTA(E37:J37)=0,$D$2,K37),WORKDAY.INTL(K37,1,$D$3))</f>
-        <v/>
-      </c>
-      <c r="M37" s="11">
-        <f>IF(D37=0,L37,WORKDAY.INTL(L37,D37-1,$D$3))</f>
-        <v/>
-      </c>
-      <c r="N37" s="9" t="n"/>
-      <c r="O37" s="10" t="inlineStr">
-        <is>
-          <t>הנחה</t>
-        </is>
-      </c>
+      <c r="A37" s="7" t="inlineStr">
+        <is>
+          <t>4. גג ופרפט</t>
+        </is>
+      </c>
+      <c r="B37" s="8" t="n"/>
+      <c r="C37" s="8" t="n"/>
+      <c r="D37" s="8" t="n"/>
+      <c r="E37" s="8" t="n"/>
+      <c r="F37" s="8" t="n"/>
+      <c r="G37" s="8" t="n"/>
+      <c r="H37" s="8" t="n"/>
+      <c r="I37" s="8" t="n"/>
+      <c r="J37" s="8" t="n"/>
+      <c r="K37" s="8" t="n"/>
+      <c r="L37" s="8" t="n"/>
+      <c r="M37" s="8" t="n"/>
+      <c r="N37" s="8" t="n"/>
+      <c r="O37" s="8" t="n"/>
+      <c r="P37" s="8" t="n"/>
+      <c r="Q37" s="8" t="n"/>
+      <c r="R37" s="8" t="n"/>
+      <c r="S37" s="8" t="n"/>
+      <c r="T37" s="8" t="n"/>
+      <c r="U37" s="8" t="n"/>
+      <c r="V37" s="8" t="n"/>
+      <c r="W37" s="8" t="n"/>
+      <c r="X37" s="8" t="n"/>
+      <c r="Y37" s="8" t="n"/>
+      <c r="Z37" s="8" t="n"/>
+      <c r="AA37" s="8" t="n"/>
+      <c r="AB37" s="8" t="n"/>
+      <c r="AC37" s="8" t="n"/>
+      <c r="AD37" s="8" t="n"/>
+      <c r="AE37" s="8" t="n"/>
+      <c r="AF37" s="8" t="n"/>
+      <c r="AG37" s="8" t="n"/>
+      <c r="AH37" s="8" t="n"/>
+      <c r="AI37" s="8" t="n"/>
+      <c r="AJ37" s="8" t="n"/>
+      <c r="AK37" s="8" t="n"/>
+      <c r="AL37" s="8" t="n"/>
+      <c r="AM37" s="8" t="n"/>
+      <c r="AN37" s="8" t="n"/>
+      <c r="AO37" s="8" t="n"/>
+      <c r="AP37" s="8" t="n"/>
+      <c r="AQ37" s="8" t="n"/>
+      <c r="AR37" s="8" t="n"/>
+      <c r="AS37" s="8" t="n"/>
+      <c r="AT37" s="8" t="n"/>
+      <c r="AU37" s="8" t="n"/>
+      <c r="AV37" s="8" t="n"/>
+      <c r="AW37" s="8" t="n"/>
+      <c r="AX37" s="8" t="n"/>
+      <c r="AY37" s="8" t="n"/>
+      <c r="AZ37" s="8" t="n"/>
+      <c r="BA37" s="8" t="n"/>
+      <c r="BB37" s="8" t="n"/>
+      <c r="BC37" s="8" t="n"/>
+      <c r="BD37" s="8" t="n"/>
+      <c r="BE37" s="8" t="n"/>
+      <c r="BF37" s="8" t="n"/>
+      <c r="BG37" s="8" t="n"/>
+      <c r="BH37" s="8" t="n"/>
+      <c r="BI37" s="8" t="n"/>
+      <c r="BJ37" s="8" t="n"/>
+      <c r="BK37" s="8" t="n"/>
+      <c r="BL37" s="8" t="n"/>
+      <c r="BM37" s="8" t="n"/>
+      <c r="BN37" s="8" t="n"/>
+      <c r="BO37" s="8" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="9" t="inlineStr">
         <is>
-          <t>R030</t>
+          <t>R010</t>
         </is>
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>בדיקת הצפה לגג (48–72 שעות) ואישור יועץ איטום</t>
+          <t>בניית פרפט חדש בהיקף הגג</t>
         </is>
       </c>
       <c r="C38" s="10" t="inlineStr">
         <is>
-          <t>11.03</t>
+          <t>11.02</t>
         </is>
       </c>
       <c r="D38" s="9" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E38" s="9" t="inlineStr">
         <is>
-          <t>R020</t>
+          <t>D070</t>
         </is>
       </c>
       <c r="F38" s="9" t="n"/>
@@ -2671,7 +2679,7 @@
       <c r="I38" s="9" t="n"/>
       <c r="J38" s="9" t="n"/>
       <c r="K38" s="11">
-        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$86,MATCH(E38,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(F38,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(G38,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(H38,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(I38,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(J38,$A$6:$A$86,0)),0))</f>
+        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$88,MATCH(E38,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(F38,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(G38,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(H38,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(I38,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(J38,$A$6:$A$88,0)),0))</f>
         <v/>
       </c>
       <c r="L38" s="11">
@@ -2685,32 +2693,32 @@
       <c r="N38" s="9" t="n"/>
       <c r="O38" s="10" t="inlineStr">
         <is>
-          <t>מפרט פרק 11</t>
+          <t>הנחה; כמות לפי מדידה</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="9" t="inlineStr">
         <is>
-          <t>R040</t>
+          <t>R020</t>
         </is>
       </c>
       <c r="B39" s="10" t="inlineStr">
         <is>
-          <t>פח קופינג וגימור פרפט</t>
+          <t>איטום גג ופרפט</t>
         </is>
       </c>
       <c r="C39" s="10" t="inlineStr">
         <is>
-          <t>11.04, 14.02</t>
+          <t>11.03</t>
         </is>
       </c>
       <c r="D39" s="9" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E39" s="9" t="inlineStr">
         <is>
-          <t>R030</t>
+          <t>R010</t>
         </is>
       </c>
       <c r="F39" s="9" t="n"/>
@@ -2719,7 +2727,7 @@
       <c r="I39" s="9" t="n"/>
       <c r="J39" s="9" t="n"/>
       <c r="K39" s="11">
-        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$86,MATCH(E39,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(F39,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(G39,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(H39,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(I39,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(J39,$A$6:$A$86,0)),0))</f>
+        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$88,MATCH(E39,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(F39,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(G39,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(H39,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(I39,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(J39,$A$6:$A$88,0)),0))</f>
         <v/>
       </c>
       <c r="L39" s="11">
@@ -2738,100 +2746,75 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="7" t="inlineStr">
-        <is>
-          <t>5. בלוקים ותשתיות מוסתרות</t>
-        </is>
-      </c>
-      <c r="B40" s="8" t="n"/>
-      <c r="C40" s="8" t="n"/>
-      <c r="D40" s="8" t="n"/>
-      <c r="E40" s="8" t="n"/>
-      <c r="F40" s="8" t="n"/>
-      <c r="G40" s="8" t="n"/>
-      <c r="H40" s="8" t="n"/>
-      <c r="I40" s="8" t="n"/>
-      <c r="J40" s="8" t="n"/>
-      <c r="K40" s="8" t="n"/>
-      <c r="L40" s="8" t="n"/>
-      <c r="M40" s="8" t="n"/>
-      <c r="N40" s="8" t="n"/>
-      <c r="O40" s="8" t="n"/>
-      <c r="P40" s="8" t="n"/>
-      <c r="Q40" s="8" t="n"/>
-      <c r="R40" s="8" t="n"/>
-      <c r="S40" s="8" t="n"/>
-      <c r="T40" s="8" t="n"/>
-      <c r="U40" s="8" t="n"/>
-      <c r="V40" s="8" t="n"/>
-      <c r="W40" s="8" t="n"/>
-      <c r="X40" s="8" t="n"/>
-      <c r="Y40" s="8" t="n"/>
-      <c r="Z40" s="8" t="n"/>
-      <c r="AA40" s="8" t="n"/>
-      <c r="AB40" s="8" t="n"/>
-      <c r="AC40" s="8" t="n"/>
-      <c r="AD40" s="8" t="n"/>
-      <c r="AE40" s="8" t="n"/>
-      <c r="AF40" s="8" t="n"/>
-      <c r="AG40" s="8" t="n"/>
-      <c r="AH40" s="8" t="n"/>
-      <c r="AI40" s="8" t="n"/>
-      <c r="AJ40" s="8" t="n"/>
-      <c r="AK40" s="8" t="n"/>
-      <c r="AL40" s="8" t="n"/>
-      <c r="AM40" s="8" t="n"/>
-      <c r="AN40" s="8" t="n"/>
-      <c r="AO40" s="8" t="n"/>
-      <c r="AP40" s="8" t="n"/>
-      <c r="AQ40" s="8" t="n"/>
-      <c r="AR40" s="8" t="n"/>
-      <c r="AS40" s="8" t="n"/>
-      <c r="AT40" s="8" t="n"/>
-      <c r="AU40" s="8" t="n"/>
-      <c r="AV40" s="8" t="n"/>
-      <c r="AW40" s="8" t="n"/>
-      <c r="AX40" s="8" t="n"/>
-      <c r="AY40" s="8" t="n"/>
-      <c r="AZ40" s="8" t="n"/>
-      <c r="BA40" s="8" t="n"/>
-      <c r="BB40" s="8" t="n"/>
-      <c r="BC40" s="8" t="n"/>
-      <c r="BD40" s="8" t="n"/>
-      <c r="BE40" s="8" t="n"/>
-      <c r="BF40" s="8" t="n"/>
-      <c r="BG40" s="8" t="n"/>
-      <c r="BH40" s="8" t="n"/>
-      <c r="BI40" s="8" t="n"/>
-      <c r="BJ40" s="8" t="n"/>
-      <c r="BK40" s="8" t="n"/>
-      <c r="BL40" s="8" t="n"/>
-      <c r="BM40" s="8" t="n"/>
-      <c r="BN40" s="8" t="n"/>
-      <c r="BO40" s="8" t="n"/>
+      <c r="A40" s="9" t="inlineStr">
+        <is>
+          <t>R030</t>
+        </is>
+      </c>
+      <c r="B40" s="10" t="inlineStr">
+        <is>
+          <t>בדיקת הצפה לגג (48–72 שעות) ואישור יועץ איטום</t>
+        </is>
+      </c>
+      <c r="C40" s="10" t="inlineStr">
+        <is>
+          <t>11.03</t>
+        </is>
+      </c>
+      <c r="D40" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="E40" s="9" t="inlineStr">
+        <is>
+          <t>R020</t>
+        </is>
+      </c>
+      <c r="F40" s="9" t="n"/>
+      <c r="G40" s="9" t="n"/>
+      <c r="H40" s="9" t="n"/>
+      <c r="I40" s="9" t="n"/>
+      <c r="J40" s="9" t="n"/>
+      <c r="K40" s="11">
+        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$88,MATCH(E40,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(F40,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(G40,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(H40,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(I40,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(J40,$A$6:$A$88,0)),0))</f>
+        <v/>
+      </c>
+      <c r="L40" s="11">
+        <f>IF(D40=0,IF(COUNTA(E40:J40)=0,$D$2,K40),WORKDAY.INTL(K40,1,$D$3))</f>
+        <v/>
+      </c>
+      <c r="M40" s="11">
+        <f>IF(D40=0,L40,WORKDAY.INTL(L40,D40-1,$D$3))</f>
+        <v/>
+      </c>
+      <c r="N40" s="9" t="n"/>
+      <c r="O40" s="10" t="inlineStr">
+        <is>
+          <t>מפרט פרק 11</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="9" t="inlineStr">
         <is>
-          <t>B010</t>
+          <t>R040</t>
         </is>
       </c>
       <c r="B41" s="10" t="inlineStr">
         <is>
-          <t>קירות בלוקים (26 מ״ר)</t>
+          <t>פח קופינג וגימור פרפט</t>
         </is>
       </c>
       <c r="C41" s="10" t="inlineStr">
         <is>
-          <t>04.01–04.03</t>
+          <t>11.04, 14.02</t>
         </is>
       </c>
       <c r="D41" s="9" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E41" s="9" t="inlineStr">
         <is>
-          <t>D070</t>
+          <t>R030</t>
         </is>
       </c>
       <c r="F41" s="9" t="n"/>
@@ -2840,7 +2823,7 @@
       <c r="I41" s="9" t="n"/>
       <c r="J41" s="9" t="n"/>
       <c r="K41" s="11">
-        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$86,MATCH(E41,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(F41,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(G41,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(H41,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(I41,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(J41,$A$6:$A$86,0)),0))</f>
+        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$88,MATCH(E41,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(F41,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(G41,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(H41,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(I41,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(J41,$A$6:$A$88,0)),0))</f>
         <v/>
       </c>
       <c r="L41" s="11">
@@ -2859,92 +2842,109 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="9" t="inlineStr">
-        <is>
-          <t>P010</t>
-        </is>
-      </c>
-      <c r="B42" s="10" t="inlineStr">
-        <is>
-          <t>אינסטלציה – נקודות, צנרת ראשית וביוב</t>
-        </is>
-      </c>
-      <c r="C42" s="10" t="inlineStr">
-        <is>
-          <t>05.25–05.33</t>
-        </is>
-      </c>
-      <c r="D42" s="9" t="n">
-        <v>20</v>
-      </c>
-      <c r="E42" s="9" t="inlineStr">
-        <is>
-          <t>D070</t>
-        </is>
-      </c>
-      <c r="F42" s="9" t="inlineStr">
-        <is>
-          <t>B010</t>
-        </is>
-      </c>
-      <c r="G42" s="9" t="n"/>
-      <c r="H42" s="9" t="n"/>
-      <c r="I42" s="9" t="n"/>
-      <c r="J42" s="9" t="n"/>
-      <c r="K42" s="11">
-        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$86,MATCH(E42,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(F42,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(G42,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(H42,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(I42,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(J42,$A$6:$A$86,0)),0))</f>
-        <v/>
-      </c>
-      <c r="L42" s="11">
-        <f>IF(D42=0,IF(COUNTA(E42:J42)=0,$D$2,K42),WORKDAY.INTL(K42,1,$D$3))</f>
-        <v/>
-      </c>
-      <c r="M42" s="11">
-        <f>IF(D42=0,L42,WORKDAY.INTL(L42,D42-1,$D$3))</f>
-        <v/>
-      </c>
-      <c r="N42" s="9" t="n"/>
-      <c r="O42" s="10" t="inlineStr">
-        <is>
-          <t>הנחה</t>
-        </is>
-      </c>
+      <c r="A42" s="7" t="inlineStr">
+        <is>
+          <t>5. בלוקים ותשתיות מוסתרות</t>
+        </is>
+      </c>
+      <c r="B42" s="8" t="n"/>
+      <c r="C42" s="8" t="n"/>
+      <c r="D42" s="8" t="n"/>
+      <c r="E42" s="8" t="n"/>
+      <c r="F42" s="8" t="n"/>
+      <c r="G42" s="8" t="n"/>
+      <c r="H42" s="8" t="n"/>
+      <c r="I42" s="8" t="n"/>
+      <c r="J42" s="8" t="n"/>
+      <c r="K42" s="8" t="n"/>
+      <c r="L42" s="8" t="n"/>
+      <c r="M42" s="8" t="n"/>
+      <c r="N42" s="8" t="n"/>
+      <c r="O42" s="8" t="n"/>
+      <c r="P42" s="8" t="n"/>
+      <c r="Q42" s="8" t="n"/>
+      <c r="R42" s="8" t="n"/>
+      <c r="S42" s="8" t="n"/>
+      <c r="T42" s="8" t="n"/>
+      <c r="U42" s="8" t="n"/>
+      <c r="V42" s="8" t="n"/>
+      <c r="W42" s="8" t="n"/>
+      <c r="X42" s="8" t="n"/>
+      <c r="Y42" s="8" t="n"/>
+      <c r="Z42" s="8" t="n"/>
+      <c r="AA42" s="8" t="n"/>
+      <c r="AB42" s="8" t="n"/>
+      <c r="AC42" s="8" t="n"/>
+      <c r="AD42" s="8" t="n"/>
+      <c r="AE42" s="8" t="n"/>
+      <c r="AF42" s="8" t="n"/>
+      <c r="AG42" s="8" t="n"/>
+      <c r="AH42" s="8" t="n"/>
+      <c r="AI42" s="8" t="n"/>
+      <c r="AJ42" s="8" t="n"/>
+      <c r="AK42" s="8" t="n"/>
+      <c r="AL42" s="8" t="n"/>
+      <c r="AM42" s="8" t="n"/>
+      <c r="AN42" s="8" t="n"/>
+      <c r="AO42" s="8" t="n"/>
+      <c r="AP42" s="8" t="n"/>
+      <c r="AQ42" s="8" t="n"/>
+      <c r="AR42" s="8" t="n"/>
+      <c r="AS42" s="8" t="n"/>
+      <c r="AT42" s="8" t="n"/>
+      <c r="AU42" s="8" t="n"/>
+      <c r="AV42" s="8" t="n"/>
+      <c r="AW42" s="8" t="n"/>
+      <c r="AX42" s="8" t="n"/>
+      <c r="AY42" s="8" t="n"/>
+      <c r="AZ42" s="8" t="n"/>
+      <c r="BA42" s="8" t="n"/>
+      <c r="BB42" s="8" t="n"/>
+      <c r="BC42" s="8" t="n"/>
+      <c r="BD42" s="8" t="n"/>
+      <c r="BE42" s="8" t="n"/>
+      <c r="BF42" s="8" t="n"/>
+      <c r="BG42" s="8" t="n"/>
+      <c r="BH42" s="8" t="n"/>
+      <c r="BI42" s="8" t="n"/>
+      <c r="BJ42" s="8" t="n"/>
+      <c r="BK42" s="8" t="n"/>
+      <c r="BL42" s="8" t="n"/>
+      <c r="BM42" s="8" t="n"/>
+      <c r="BN42" s="8" t="n"/>
+      <c r="BO42" s="8" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="9" t="inlineStr">
         <is>
-          <t>E010</t>
+          <t>B010</t>
         </is>
       </c>
       <c r="B43" s="10" t="inlineStr">
         <is>
-          <t>חשמל ותאורה – צנרת, שרוולים, נקודות ולוחות</t>
+          <t>קירות בלוקים (26 מ״ר)</t>
         </is>
       </c>
       <c r="C43" s="10" t="inlineStr">
         <is>
-          <t>06, 07.20</t>
+          <t>04.01–04.03</t>
         </is>
       </c>
       <c r="D43" s="9" t="n">
-        <v>20</v>
+        <v>4</v>
       </c>
       <c r="E43" s="9" t="inlineStr">
         <is>
           <t>D070</t>
         </is>
       </c>
-      <c r="F43" s="9" t="inlineStr">
-        <is>
-          <t>B010</t>
-        </is>
-      </c>
+      <c r="F43" s="9" t="n"/>
       <c r="G43" s="9" t="n"/>
       <c r="H43" s="9" t="n"/>
       <c r="I43" s="9" t="n"/>
       <c r="J43" s="9" t="n"/>
       <c r="K43" s="11">
-        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$86,MATCH(E43,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(F43,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(G43,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(H43,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(I43,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(J43,$A$6:$A$86,0)),0))</f>
+        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$88,MATCH(E43,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(F43,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(G43,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(H43,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(I43,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(J43,$A$6:$A$88,0)),0))</f>
         <v/>
       </c>
       <c r="L43" s="11">
@@ -2965,30 +2965,30 @@
     <row r="44">
       <c r="A44" s="9" t="inlineStr">
         <is>
-          <t>M010</t>
+          <t>P010</t>
         </is>
       </c>
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t>צנרת קירור וניקוז למיזוג</t>
+          <t>אינסטלציה – נקודות, צנרת ראשית וביוב</t>
         </is>
       </c>
       <c r="C44" s="10" t="inlineStr">
         <is>
-          <t>08.02</t>
+          <t>05.25–05.33</t>
         </is>
       </c>
       <c r="D44" s="9" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="E44" s="9" t="inlineStr">
         <is>
+          <t>D070</t>
+        </is>
+      </c>
+      <c r="F44" s="9" t="inlineStr">
+        <is>
           <t>B010</t>
-        </is>
-      </c>
-      <c r="F44" s="9" t="inlineStr">
-        <is>
-          <t>A065</t>
         </is>
       </c>
       <c r="G44" s="9" t="n"/>
@@ -2996,7 +2996,7 @@
       <c r="I44" s="9" t="n"/>
       <c r="J44" s="9" t="n"/>
       <c r="K44" s="11">
-        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$86,MATCH(E44,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(F44,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(G44,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(H44,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(I44,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(J44,$A$6:$A$86,0)),0))</f>
+        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$88,MATCH(E44,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(F44,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(G44,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(H44,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(I44,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(J44,$A$6:$A$88,0)),0))</f>
         <v/>
       </c>
       <c r="L44" s="11">
@@ -3017,34 +3017,38 @@
     <row r="45">
       <c r="A45" s="9" t="inlineStr">
         <is>
-          <t>C010</t>
+          <t>E010</t>
         </is>
       </c>
       <c r="B45" s="10" t="inlineStr">
         <is>
-          <t>צנרת ושרוולים לתקשורת, מיגון ושמע</t>
+          <t>חשמל ותאורה – צנרת, שרוולים, נקודות ולוחות</t>
         </is>
       </c>
       <c r="C45" s="10" t="inlineStr">
         <is>
-          <t>18.01</t>
+          <t>06, 07.20</t>
         </is>
       </c>
       <c r="D45" s="9" t="n">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="E45" s="9" t="inlineStr">
         <is>
+          <t>D070</t>
+        </is>
+      </c>
+      <c r="F45" s="9" t="inlineStr">
+        <is>
           <t>B010</t>
         </is>
       </c>
-      <c r="F45" s="9" t="n"/>
       <c r="G45" s="9" t="n"/>
       <c r="H45" s="9" t="n"/>
       <c r="I45" s="9" t="n"/>
       <c r="J45" s="9" t="n"/>
       <c r="K45" s="11">
-        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$86,MATCH(E45,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(F45,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(G45,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(H45,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(I45,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(J45,$A$6:$A$86,0)),0))</f>
+        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$88,MATCH(E45,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(F45,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(G45,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(H45,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(I45,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(J45,$A$6:$A$88,0)),0))</f>
         <v/>
       </c>
       <c r="L45" s="11">
@@ -3065,34 +3069,38 @@
     <row r="46">
       <c r="A46" s="9" t="inlineStr">
         <is>
-          <t>Q010</t>
+          <t>M010</t>
         </is>
       </c>
       <c r="B46" s="10" t="inlineStr">
         <is>
-          <t>בדיקות לחץ ואטימות אינסטלציה ואישור מתכננת</t>
+          <t>צנרת קירור וניקוז למיזוג</t>
         </is>
       </c>
       <c r="C46" s="10" t="inlineStr">
         <is>
-          <t>05.35</t>
+          <t>08.02</t>
         </is>
       </c>
       <c r="D46" s="9" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E46" s="9" t="inlineStr">
         <is>
-          <t>P010</t>
-        </is>
-      </c>
-      <c r="F46" s="9" t="n"/>
+          <t>B010</t>
+        </is>
+      </c>
+      <c r="F46" s="9" t="inlineStr">
+        <is>
+          <t>A065</t>
+        </is>
+      </c>
       <c r="G46" s="9" t="n"/>
       <c r="H46" s="9" t="n"/>
       <c r="I46" s="9" t="n"/>
       <c r="J46" s="9" t="n"/>
       <c r="K46" s="11">
-        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$86,MATCH(E46,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(F46,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(G46,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(H46,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(I46,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(J46,$A$6:$A$86,0)),0))</f>
+        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$88,MATCH(E46,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(F46,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(G46,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(H46,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(I46,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(J46,$A$6:$A$88,0)),0))</f>
         <v/>
       </c>
       <c r="L46" s="11">
@@ -3106,32 +3114,32 @@
       <c r="N46" s="9" t="n"/>
       <c r="O46" s="10" t="inlineStr">
         <is>
-          <t>מפרט פרק 5</t>
+          <t>הנחה</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="9" t="inlineStr">
         <is>
-          <t>Q020</t>
+          <t>C010</t>
         </is>
       </c>
       <c r="B47" s="10" t="inlineStr">
         <is>
-          <t>בדיקת חשמלאי בודק לתשתיות, הארקה ופחת</t>
+          <t>צנרת ושרוולים לתקשורת, מיגון ושמע</t>
         </is>
       </c>
       <c r="C47" s="10" t="inlineStr">
         <is>
-          <t>06.09</t>
+          <t>18.01</t>
         </is>
       </c>
       <c r="D47" s="9" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E47" s="9" t="inlineStr">
         <is>
-          <t>E010</t>
+          <t>B010</t>
         </is>
       </c>
       <c r="F47" s="9" t="n"/>
@@ -3140,7 +3148,7 @@
       <c r="I47" s="9" t="n"/>
       <c r="J47" s="9" t="n"/>
       <c r="K47" s="11">
-        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$86,MATCH(E47,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(F47,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(G47,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(H47,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(I47,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(J47,$A$6:$A$86,0)),0))</f>
+        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$88,MATCH(E47,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(F47,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(G47,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(H47,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(I47,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(J47,$A$6:$A$88,0)),0))</f>
         <v/>
       </c>
       <c r="L47" s="11">
@@ -3154,130 +3162,89 @@
       <c r="N47" s="9" t="n"/>
       <c r="O47" s="10" t="inlineStr">
         <is>
-          <t>מפרט פרק 6</t>
+          <t>הנחה</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="7" t="inlineStr">
-        <is>
-          <t>6. גבס ואיטום פנים</t>
-        </is>
-      </c>
-      <c r="B48" s="8" t="n"/>
-      <c r="C48" s="8" t="n"/>
-      <c r="D48" s="8" t="n"/>
-      <c r="E48" s="8" t="n"/>
-      <c r="F48" s="8" t="n"/>
-      <c r="G48" s="8" t="n"/>
-      <c r="H48" s="8" t="n"/>
-      <c r="I48" s="8" t="n"/>
-      <c r="J48" s="8" t="n"/>
-      <c r="K48" s="8" t="n"/>
-      <c r="L48" s="8" t="n"/>
-      <c r="M48" s="8" t="n"/>
-      <c r="N48" s="8" t="n"/>
-      <c r="O48" s="8" t="n"/>
-      <c r="P48" s="8" t="n"/>
-      <c r="Q48" s="8" t="n"/>
-      <c r="R48" s="8" t="n"/>
-      <c r="S48" s="8" t="n"/>
-      <c r="T48" s="8" t="n"/>
-      <c r="U48" s="8" t="n"/>
-      <c r="V48" s="8" t="n"/>
-      <c r="W48" s="8" t="n"/>
-      <c r="X48" s="8" t="n"/>
-      <c r="Y48" s="8" t="n"/>
-      <c r="Z48" s="8" t="n"/>
-      <c r="AA48" s="8" t="n"/>
-      <c r="AB48" s="8" t="n"/>
-      <c r="AC48" s="8" t="n"/>
-      <c r="AD48" s="8" t="n"/>
-      <c r="AE48" s="8" t="n"/>
-      <c r="AF48" s="8" t="n"/>
-      <c r="AG48" s="8" t="n"/>
-      <c r="AH48" s="8" t="n"/>
-      <c r="AI48" s="8" t="n"/>
-      <c r="AJ48" s="8" t="n"/>
-      <c r="AK48" s="8" t="n"/>
-      <c r="AL48" s="8" t="n"/>
-      <c r="AM48" s="8" t="n"/>
-      <c r="AN48" s="8" t="n"/>
-      <c r="AO48" s="8" t="n"/>
-      <c r="AP48" s="8" t="n"/>
-      <c r="AQ48" s="8" t="n"/>
-      <c r="AR48" s="8" t="n"/>
-      <c r="AS48" s="8" t="n"/>
-      <c r="AT48" s="8" t="n"/>
-      <c r="AU48" s="8" t="n"/>
-      <c r="AV48" s="8" t="n"/>
-      <c r="AW48" s="8" t="n"/>
-      <c r="AX48" s="8" t="n"/>
-      <c r="AY48" s="8" t="n"/>
-      <c r="AZ48" s="8" t="n"/>
-      <c r="BA48" s="8" t="n"/>
-      <c r="BB48" s="8" t="n"/>
-      <c r="BC48" s="8" t="n"/>
-      <c r="BD48" s="8" t="n"/>
-      <c r="BE48" s="8" t="n"/>
-      <c r="BF48" s="8" t="n"/>
-      <c r="BG48" s="8" t="n"/>
-      <c r="BH48" s="8" t="n"/>
-      <c r="BI48" s="8" t="n"/>
-      <c r="BJ48" s="8" t="n"/>
-      <c r="BK48" s="8" t="n"/>
-      <c r="BL48" s="8" t="n"/>
-      <c r="BM48" s="8" t="n"/>
-      <c r="BN48" s="8" t="n"/>
-      <c r="BO48" s="8" t="n"/>
+      <c r="A48" s="9" t="inlineStr">
+        <is>
+          <t>Q010</t>
+        </is>
+      </c>
+      <c r="B48" s="10" t="inlineStr">
+        <is>
+          <t>בדיקות לחץ ואטימות אינסטלציה ואישור מתכננת</t>
+        </is>
+      </c>
+      <c r="C48" s="10" t="inlineStr">
+        <is>
+          <t>05.35</t>
+        </is>
+      </c>
+      <c r="D48" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="E48" s="9" t="inlineStr">
+        <is>
+          <t>P010</t>
+        </is>
+      </c>
+      <c r="F48" s="9" t="n"/>
+      <c r="G48" s="9" t="n"/>
+      <c r="H48" s="9" t="n"/>
+      <c r="I48" s="9" t="n"/>
+      <c r="J48" s="9" t="n"/>
+      <c r="K48" s="11">
+        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$88,MATCH(E48,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(F48,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(G48,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(H48,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(I48,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(J48,$A$6:$A$88,0)),0))</f>
+        <v/>
+      </c>
+      <c r="L48" s="11">
+        <f>IF(D48=0,IF(COUNTA(E48:J48)=0,$D$2,K48),WORKDAY.INTL(K48,1,$D$3))</f>
+        <v/>
+      </c>
+      <c r="M48" s="11">
+        <f>IF(D48=0,L48,WORKDAY.INTL(L48,D48-1,$D$3))</f>
+        <v/>
+      </c>
+      <c r="N48" s="9" t="n"/>
+      <c r="O48" s="10" t="inlineStr">
+        <is>
+          <t>מפרט פרק 5</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="9" t="inlineStr">
         <is>
-          <t>G010</t>
+          <t>Q020</t>
         </is>
       </c>
       <c r="B49" s="10" t="inlineStr">
         <is>
-          <t>מחיצות גבס כולל בידוד אקוסטי (133 מ״ר)</t>
+          <t>בדיקת חשמלאי בודק לתשתיות, הארקה ופחת</t>
         </is>
       </c>
       <c r="C49" s="10" t="inlineStr">
         <is>
-          <t>09.01–09.03</t>
+          <t>06.09</t>
         </is>
       </c>
       <c r="D49" s="9" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="E49" s="9" t="inlineStr">
         <is>
-          <t>Q010</t>
-        </is>
-      </c>
-      <c r="F49" s="9" t="inlineStr">
-        <is>
-          <t>Q020</t>
-        </is>
-      </c>
-      <c r="G49" s="9" t="inlineStr">
-        <is>
-          <t>M010</t>
-        </is>
-      </c>
-      <c r="H49" s="9" t="inlineStr">
-        <is>
-          <t>C010</t>
-        </is>
-      </c>
-      <c r="I49" s="9" t="inlineStr">
-        <is>
-          <t>K050</t>
-        </is>
-      </c>
+          <t>E010</t>
+        </is>
+      </c>
+      <c r="F49" s="9" t="n"/>
+      <c r="G49" s="9" t="n"/>
+      <c r="H49" s="9" t="n"/>
+      <c r="I49" s="9" t="n"/>
       <c r="J49" s="9" t="n"/>
       <c r="K49" s="11">
-        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$86,MATCH(E49,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(F49,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(G49,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(H49,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(I49,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(J49,$A$6:$A$86,0)),0))</f>
+        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$88,MATCH(E49,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(F49,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(G49,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(H49,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(I49,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(J49,$A$6:$A$88,0)),0))</f>
         <v/>
       </c>
       <c r="L49" s="11">
@@ -3288,100 +3255,133 @@
         <f>IF(D49=0,L49,WORKDAY.INTL(L49,D49-1,$D$3))</f>
         <v/>
       </c>
-      <c r="N49" s="12" t="inlineStr">
-        <is>
-          <t>כן</t>
-        </is>
-      </c>
+      <c r="N49" s="9" t="n"/>
       <c r="O49" s="10" t="inlineStr">
         <is>
-          <t>הנחה: ~11 מ״ר ליום</t>
+          <t>מפרט פרק 6</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="9" t="inlineStr">
-        <is>
-          <t>G020</t>
-        </is>
-      </c>
-      <c r="B50" s="10" t="inlineStr">
-        <is>
-          <t>תקרות גבס תלויות (33.3 מ״ר) ופתחי תאורה</t>
-        </is>
-      </c>
-      <c r="C50" s="10" t="inlineStr">
-        <is>
-          <t>09.04</t>
-        </is>
-      </c>
-      <c r="D50" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="E50" s="9" t="inlineStr">
-        <is>
-          <t>G010</t>
-        </is>
-      </c>
-      <c r="F50" s="9" t="n"/>
-      <c r="G50" s="9" t="n"/>
-      <c r="H50" s="9" t="n"/>
-      <c r="I50" s="9" t="n"/>
-      <c r="J50" s="9" t="n"/>
-      <c r="K50" s="11">
-        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$86,MATCH(E50,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(F50,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(G50,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(H50,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(I50,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(J50,$A$6:$A$86,0)),0))</f>
-        <v/>
-      </c>
-      <c r="L50" s="11">
-        <f>IF(D50=0,IF(COUNTA(E50:J50)=0,$D$2,K50),WORKDAY.INTL(K50,1,$D$3))</f>
-        <v/>
-      </c>
-      <c r="M50" s="11">
-        <f>IF(D50=0,L50,WORKDAY.INTL(L50,D50-1,$D$3))</f>
-        <v/>
-      </c>
-      <c r="N50" s="12" t="inlineStr">
-        <is>
-          <t>כן</t>
-        </is>
-      </c>
-      <c r="O50" s="10" t="inlineStr">
-        <is>
-          <t>הנחה</t>
-        </is>
-      </c>
+      <c r="A50" s="7" t="inlineStr">
+        <is>
+          <t>6. גבס ואיטום פנים</t>
+        </is>
+      </c>
+      <c r="B50" s="8" t="n"/>
+      <c r="C50" s="8" t="n"/>
+      <c r="D50" s="8" t="n"/>
+      <c r="E50" s="8" t="n"/>
+      <c r="F50" s="8" t="n"/>
+      <c r="G50" s="8" t="n"/>
+      <c r="H50" s="8" t="n"/>
+      <c r="I50" s="8" t="n"/>
+      <c r="J50" s="8" t="n"/>
+      <c r="K50" s="8" t="n"/>
+      <c r="L50" s="8" t="n"/>
+      <c r="M50" s="8" t="n"/>
+      <c r="N50" s="8" t="n"/>
+      <c r="O50" s="8" t="n"/>
+      <c r="P50" s="8" t="n"/>
+      <c r="Q50" s="8" t="n"/>
+      <c r="R50" s="8" t="n"/>
+      <c r="S50" s="8" t="n"/>
+      <c r="T50" s="8" t="n"/>
+      <c r="U50" s="8" t="n"/>
+      <c r="V50" s="8" t="n"/>
+      <c r="W50" s="8" t="n"/>
+      <c r="X50" s="8" t="n"/>
+      <c r="Y50" s="8" t="n"/>
+      <c r="Z50" s="8" t="n"/>
+      <c r="AA50" s="8" t="n"/>
+      <c r="AB50" s="8" t="n"/>
+      <c r="AC50" s="8" t="n"/>
+      <c r="AD50" s="8" t="n"/>
+      <c r="AE50" s="8" t="n"/>
+      <c r="AF50" s="8" t="n"/>
+      <c r="AG50" s="8" t="n"/>
+      <c r="AH50" s="8" t="n"/>
+      <c r="AI50" s="8" t="n"/>
+      <c r="AJ50" s="8" t="n"/>
+      <c r="AK50" s="8" t="n"/>
+      <c r="AL50" s="8" t="n"/>
+      <c r="AM50" s="8" t="n"/>
+      <c r="AN50" s="8" t="n"/>
+      <c r="AO50" s="8" t="n"/>
+      <c r="AP50" s="8" t="n"/>
+      <c r="AQ50" s="8" t="n"/>
+      <c r="AR50" s="8" t="n"/>
+      <c r="AS50" s="8" t="n"/>
+      <c r="AT50" s="8" t="n"/>
+      <c r="AU50" s="8" t="n"/>
+      <c r="AV50" s="8" t="n"/>
+      <c r="AW50" s="8" t="n"/>
+      <c r="AX50" s="8" t="n"/>
+      <c r="AY50" s="8" t="n"/>
+      <c r="AZ50" s="8" t="n"/>
+      <c r="BA50" s="8" t="n"/>
+      <c r="BB50" s="8" t="n"/>
+      <c r="BC50" s="8" t="n"/>
+      <c r="BD50" s="8" t="n"/>
+      <c r="BE50" s="8" t="n"/>
+      <c r="BF50" s="8" t="n"/>
+      <c r="BG50" s="8" t="n"/>
+      <c r="BH50" s="8" t="n"/>
+      <c r="BI50" s="8" t="n"/>
+      <c r="BJ50" s="8" t="n"/>
+      <c r="BK50" s="8" t="n"/>
+      <c r="BL50" s="8" t="n"/>
+      <c r="BM50" s="8" t="n"/>
+      <c r="BN50" s="8" t="n"/>
+      <c r="BO50" s="8" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="9" t="inlineStr">
         <is>
-          <t>G030</t>
+          <t>G010</t>
         </is>
       </c>
       <c r="B51" s="10" t="inlineStr">
         <is>
-          <t>בדיקת גבס ואישור לניצבות ותשתיות</t>
+          <t>מחיצות גבס כולל בידוד אקוסטי (133 מ״ר)</t>
         </is>
       </c>
       <c r="C51" s="10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>09.01–09.03</t>
         </is>
       </c>
       <c r="D51" s="9" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="E51" s="9" t="inlineStr">
         <is>
-          <t>G020</t>
-        </is>
-      </c>
-      <c r="F51" s="9" t="n"/>
-      <c r="G51" s="9" t="n"/>
-      <c r="H51" s="9" t="n"/>
-      <c r="I51" s="9" t="n"/>
+          <t>Q010</t>
+        </is>
+      </c>
+      <c r="F51" s="9" t="inlineStr">
+        <is>
+          <t>Q020</t>
+        </is>
+      </c>
+      <c r="G51" s="9" t="inlineStr">
+        <is>
+          <t>M010</t>
+        </is>
+      </c>
+      <c r="H51" s="9" t="inlineStr">
+        <is>
+          <t>C010</t>
+        </is>
+      </c>
+      <c r="I51" s="9" t="inlineStr">
+        <is>
+          <t>K050</t>
+        </is>
+      </c>
       <c r="J51" s="9" t="n"/>
       <c r="K51" s="11">
-        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$86,MATCH(E51,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(F51,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(G51,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(H51,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(I51,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(J51,$A$6:$A$86,0)),0))</f>
+        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$88,MATCH(E51,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(F51,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(G51,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(H51,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(I51,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(J51,$A$6:$A$88,0)),0))</f>
         <v/>
       </c>
       <c r="L51" s="11">
@@ -3399,45 +3399,41 @@
       </c>
       <c r="O51" s="10" t="inlineStr">
         <is>
-          <t>מפרט פרק 9</t>
+          <t>הנחה: ~11 מ״ר ליום</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="9" t="inlineStr">
         <is>
-          <t>W010</t>
+          <t>G020</t>
         </is>
       </c>
       <c r="B52" s="10" t="inlineStr">
         <is>
-          <t>איטום רצפות וקירות חדרים רטובים (226 מ״ר)</t>
+          <t>תקרות גבס תלויות (33.3 מ״ר) ופתחי תאורה</t>
         </is>
       </c>
       <c r="C52" s="10" t="inlineStr">
         <is>
-          <t>10.01, 10.02</t>
+          <t>09.04</t>
         </is>
       </c>
       <c r="D52" s="9" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E52" s="9" t="inlineStr">
         <is>
-          <t>Q010</t>
-        </is>
-      </c>
-      <c r="F52" s="9" t="inlineStr">
-        <is>
-          <t>B010</t>
-        </is>
-      </c>
+          <t>G010</t>
+        </is>
+      </c>
+      <c r="F52" s="9" t="n"/>
       <c r="G52" s="9" t="n"/>
       <c r="H52" s="9" t="n"/>
       <c r="I52" s="9" t="n"/>
       <c r="J52" s="9" t="n"/>
       <c r="K52" s="11">
-        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$86,MATCH(E52,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(F52,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(G52,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(H52,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(I52,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(J52,$A$6:$A$86,0)),0))</f>
+        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$88,MATCH(E52,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(F52,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(G52,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(H52,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(I52,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(J52,$A$6:$A$88,0)),0))</f>
         <v/>
       </c>
       <c r="L52" s="11">
@@ -3448,7 +3444,11 @@
         <f>IF(D52=0,L52,WORKDAY.INTL(L52,D52-1,$D$3))</f>
         <v/>
       </c>
-      <c r="N52" s="9" t="n"/>
+      <c r="N52" s="12" t="inlineStr">
+        <is>
+          <t>כן</t>
+        </is>
+      </c>
       <c r="O52" s="10" t="inlineStr">
         <is>
           <t>הנחה</t>
@@ -3458,38 +3458,34 @@
     <row r="53">
       <c r="A53" s="9" t="inlineStr">
         <is>
-          <t>W020</t>
+          <t>G030</t>
         </is>
       </c>
       <c r="B53" s="10" t="inlineStr">
         <is>
-          <t>איטום מרפסות (52.7 מ״ר)</t>
+          <t>בדיקת גבס ואישור לניצבות ותשתיות</t>
         </is>
       </c>
       <c r="C53" s="10" t="inlineStr">
         <is>
-          <t>10.04</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D53" s="9" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E53" s="9" t="inlineStr">
         <is>
-          <t>K030</t>
-        </is>
-      </c>
-      <c r="F53" s="9" t="inlineStr">
-        <is>
-          <t>Q010</t>
-        </is>
-      </c>
+          <t>G020</t>
+        </is>
+      </c>
+      <c r="F53" s="9" t="n"/>
       <c r="G53" s="9" t="n"/>
       <c r="H53" s="9" t="n"/>
       <c r="I53" s="9" t="n"/>
       <c r="J53" s="9" t="n"/>
       <c r="K53" s="11">
-        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$86,MATCH(E53,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(F53,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(G53,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(H53,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(I53,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(J53,$A$6:$A$86,0)),0))</f>
+        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$88,MATCH(E53,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(F53,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(G53,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(H53,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(I53,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(J53,$A$6:$A$88,0)),0))</f>
         <v/>
       </c>
       <c r="L53" s="11">
@@ -3500,40 +3496,44 @@
         <f>IF(D53=0,L53,WORKDAY.INTL(L53,D53-1,$D$3))</f>
         <v/>
       </c>
-      <c r="N53" s="9" t="n"/>
+      <c r="N53" s="12" t="inlineStr">
+        <is>
+          <t>כן</t>
+        </is>
+      </c>
       <c r="O53" s="10" t="inlineStr">
         <is>
-          <t>הנחה</t>
+          <t>מפרט פרק 9</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="9" t="inlineStr">
         <is>
-          <t>W030</t>
+          <t>W010</t>
         </is>
       </c>
       <c r="B54" s="10" t="inlineStr">
         <is>
-          <t>בדיקות הצפה לחדרים רטובים ולמרפסות (48–72 שעות)</t>
+          <t>איטום רצפות וקירות חדרים רטובים (226 מ״ר)</t>
         </is>
       </c>
       <c r="C54" s="10" t="inlineStr">
         <is>
-          <t>10.03</t>
+          <t>10.01, 10.02</t>
         </is>
       </c>
       <c r="D54" s="9" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="E54" s="9" t="inlineStr">
         <is>
-          <t>W010</t>
+          <t>Q010</t>
         </is>
       </c>
       <c r="F54" s="9" t="inlineStr">
         <is>
-          <t>W020</t>
+          <t>B010</t>
         </is>
       </c>
       <c r="G54" s="9" t="n"/>
@@ -3541,7 +3541,7 @@
       <c r="I54" s="9" t="n"/>
       <c r="J54" s="9" t="n"/>
       <c r="K54" s="11">
-        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$86,MATCH(E54,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(F54,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(G54,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(H54,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(I54,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(J54,$A$6:$A$86,0)),0))</f>
+        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$88,MATCH(E54,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(F54,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(G54,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(H54,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(I54,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(J54,$A$6:$A$88,0)),0))</f>
         <v/>
       </c>
       <c r="L54" s="11">
@@ -3555,41 +3555,45 @@
       <c r="N54" s="9" t="n"/>
       <c r="O54" s="10" t="inlineStr">
         <is>
-          <t>מפרט פרק 10</t>
+          <t>הנחה</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="9" t="inlineStr">
         <is>
-          <t>W040</t>
+          <t>W020</t>
         </is>
       </c>
       <c r="B55" s="10" t="inlineStr">
         <is>
-          <t>אישור יועץ האיטום בכתב</t>
+          <t>איטום מרפסות (52.7 מ״ר)</t>
         </is>
       </c>
       <c r="C55" s="10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>10.04</t>
         </is>
       </c>
       <c r="D55" s="9" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E55" s="9" t="inlineStr">
         <is>
-          <t>W030</t>
-        </is>
-      </c>
-      <c r="F55" s="9" t="n"/>
+          <t>K030</t>
+        </is>
+      </c>
+      <c r="F55" s="9" t="inlineStr">
+        <is>
+          <t>Q010</t>
+        </is>
+      </c>
       <c r="G55" s="9" t="n"/>
       <c r="H55" s="9" t="n"/>
       <c r="I55" s="9" t="n"/>
       <c r="J55" s="9" t="n"/>
       <c r="K55" s="11">
-        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$86,MATCH(E55,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(F55,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(G55,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(H55,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(I55,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(J55,$A$6:$A$86,0)),0))</f>
+        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$88,MATCH(E55,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(F55,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(G55,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(H55,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(I55,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(J55,$A$6:$A$88,0)),0))</f>
         <v/>
       </c>
       <c r="L55" s="11">
@@ -3603,105 +3607,84 @@
       <c r="N55" s="9" t="n"/>
       <c r="O55" s="10" t="inlineStr">
         <is>
+          <t>הנחה</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="9" t="inlineStr">
+        <is>
+          <t>W030</t>
+        </is>
+      </c>
+      <c r="B56" s="10" t="inlineStr">
+        <is>
+          <t>בדיקות הצפה לחדרים רטובים ולמרפסות (48–72 שעות)</t>
+        </is>
+      </c>
+      <c r="C56" s="10" t="inlineStr">
+        <is>
+          <t>10.03</t>
+        </is>
+      </c>
+      <c r="D56" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="E56" s="9" t="inlineStr">
+        <is>
+          <t>W010</t>
+        </is>
+      </c>
+      <c r="F56" s="9" t="inlineStr">
+        <is>
+          <t>W020</t>
+        </is>
+      </c>
+      <c r="G56" s="9" t="n"/>
+      <c r="H56" s="9" t="n"/>
+      <c r="I56" s="9" t="n"/>
+      <c r="J56" s="9" t="n"/>
+      <c r="K56" s="11">
+        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$88,MATCH(E56,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(F56,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(G56,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(H56,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(I56,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(J56,$A$6:$A$88,0)),0))</f>
+        <v/>
+      </c>
+      <c r="L56" s="11">
+        <f>IF(D56=0,IF(COUNTA(E56:J56)=0,$D$2,K56),WORKDAY.INTL(K56,1,$D$3))</f>
+        <v/>
+      </c>
+      <c r="M56" s="11">
+        <f>IF(D56=0,L56,WORKDAY.INTL(L56,D56-1,$D$3))</f>
+        <v/>
+      </c>
+      <c r="N56" s="9" t="n"/>
+      <c r="O56" s="10" t="inlineStr">
+        <is>
           <t>מפרט פרק 10</t>
         </is>
       </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="7" t="inlineStr">
-        <is>
-          <t>7. חזית ושלד חיצוני (במקביל)</t>
-        </is>
-      </c>
-      <c r="B56" s="8" t="n"/>
-      <c r="C56" s="8" t="n"/>
-      <c r="D56" s="8" t="n"/>
-      <c r="E56" s="8" t="n"/>
-      <c r="F56" s="8" t="n"/>
-      <c r="G56" s="8" t="n"/>
-      <c r="H56" s="8" t="n"/>
-      <c r="I56" s="8" t="n"/>
-      <c r="J56" s="8" t="n"/>
-      <c r="K56" s="8" t="n"/>
-      <c r="L56" s="8" t="n"/>
-      <c r="M56" s="8" t="n"/>
-      <c r="N56" s="8" t="n"/>
-      <c r="O56" s="8" t="n"/>
-      <c r="P56" s="8" t="n"/>
-      <c r="Q56" s="8" t="n"/>
-      <c r="R56" s="8" t="n"/>
-      <c r="S56" s="8" t="n"/>
-      <c r="T56" s="8" t="n"/>
-      <c r="U56" s="8" t="n"/>
-      <c r="V56" s="8" t="n"/>
-      <c r="W56" s="8" t="n"/>
-      <c r="X56" s="8" t="n"/>
-      <c r="Y56" s="8" t="n"/>
-      <c r="Z56" s="8" t="n"/>
-      <c r="AA56" s="8" t="n"/>
-      <c r="AB56" s="8" t="n"/>
-      <c r="AC56" s="8" t="n"/>
-      <c r="AD56" s="8" t="n"/>
-      <c r="AE56" s="8" t="n"/>
-      <c r="AF56" s="8" t="n"/>
-      <c r="AG56" s="8" t="n"/>
-      <c r="AH56" s="8" t="n"/>
-      <c r="AI56" s="8" t="n"/>
-      <c r="AJ56" s="8" t="n"/>
-      <c r="AK56" s="8" t="n"/>
-      <c r="AL56" s="8" t="n"/>
-      <c r="AM56" s="8" t="n"/>
-      <c r="AN56" s="8" t="n"/>
-      <c r="AO56" s="8" t="n"/>
-      <c r="AP56" s="8" t="n"/>
-      <c r="AQ56" s="8" t="n"/>
-      <c r="AR56" s="8" t="n"/>
-      <c r="AS56" s="8" t="n"/>
-      <c r="AT56" s="8" t="n"/>
-      <c r="AU56" s="8" t="n"/>
-      <c r="AV56" s="8" t="n"/>
-      <c r="AW56" s="8" t="n"/>
-      <c r="AX56" s="8" t="n"/>
-      <c r="AY56" s="8" t="n"/>
-      <c r="AZ56" s="8" t="n"/>
-      <c r="BA56" s="8" t="n"/>
-      <c r="BB56" s="8" t="n"/>
-      <c r="BC56" s="8" t="n"/>
-      <c r="BD56" s="8" t="n"/>
-      <c r="BE56" s="8" t="n"/>
-      <c r="BF56" s="8" t="n"/>
-      <c r="BG56" s="8" t="n"/>
-      <c r="BH56" s="8" t="n"/>
-      <c r="BI56" s="8" t="n"/>
-      <c r="BJ56" s="8" t="n"/>
-      <c r="BK56" s="8" t="n"/>
-      <c r="BL56" s="8" t="n"/>
-      <c r="BM56" s="8" t="n"/>
-      <c r="BN56" s="8" t="n"/>
-      <c r="BO56" s="8" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="9" t="inlineStr">
         <is>
-          <t>X010</t>
+          <t>W040</t>
         </is>
       </c>
       <c r="B57" s="10" t="inlineStr">
         <is>
-          <t>הקמת פיגומים</t>
+          <t>אישור יועץ האיטום בכתב</t>
         </is>
       </c>
       <c r="C57" s="10" t="inlineStr">
         <is>
-          <t>14.01</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D57" s="9" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E57" s="9" t="inlineStr">
         <is>
-          <t>D070</t>
+          <t>W030</t>
         </is>
       </c>
       <c r="F57" s="9" t="n"/>
@@ -3710,7 +3693,7 @@
       <c r="I57" s="9" t="n"/>
       <c r="J57" s="9" t="n"/>
       <c r="K57" s="11">
-        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$86,MATCH(E57,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(F57,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(G57,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(H57,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(I57,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(J57,$A$6:$A$86,0)),0))</f>
+        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$88,MATCH(E57,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(F57,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(G57,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(H57,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(I57,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(J57,$A$6:$A$88,0)),0))</f>
         <v/>
       </c>
       <c r="L57" s="11">
@@ -3724,101 +3707,118 @@
       <c r="N57" s="9" t="n"/>
       <c r="O57" s="10" t="inlineStr">
         <is>
-          <t>הנחה</t>
+          <t>מפרט פרק 10</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="9" t="inlineStr">
-        <is>
-          <t>L010</t>
-        </is>
-      </c>
-      <c r="B58" s="10" t="inlineStr">
-        <is>
-          <t>התקנת אלומיניום – חלונות ודלתות חוץ (26 יח׳)</t>
-        </is>
-      </c>
-      <c r="C58" s="10" t="inlineStr">
-        <is>
-          <t>16.01</t>
-        </is>
-      </c>
-      <c r="D58" s="9" t="n">
-        <v>10</v>
-      </c>
-      <c r="E58" s="9" t="inlineStr">
-        <is>
-          <t>A045</t>
-        </is>
-      </c>
-      <c r="F58" s="9" t="inlineStr">
-        <is>
-          <t>K050</t>
-        </is>
-      </c>
-      <c r="G58" s="9" t="n"/>
-      <c r="H58" s="9" t="n"/>
-      <c r="I58" s="9" t="n"/>
-      <c r="J58" s="9" t="n"/>
-      <c r="K58" s="11">
-        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$86,MATCH(E58,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(F58,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(G58,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(H58,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(I58,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(J58,$A$6:$A$86,0)),0))</f>
-        <v/>
-      </c>
-      <c r="L58" s="11">
-        <f>IF(D58=0,IF(COUNTA(E58:J58)=0,$D$2,K58),WORKDAY.INTL(K58,1,$D$3))</f>
-        <v/>
-      </c>
-      <c r="M58" s="11">
-        <f>IF(D58=0,L58,WORKDAY.INTL(L58,D58-1,$D$3))</f>
-        <v/>
-      </c>
-      <c r="N58" s="9" t="n"/>
-      <c r="O58" s="10" t="inlineStr">
-        <is>
-          <t>הנחה</t>
-        </is>
-      </c>
+      <c r="A58" s="7" t="inlineStr">
+        <is>
+          <t>7. חזית ושלד חיצוני (במקביל)</t>
+        </is>
+      </c>
+      <c r="B58" s="8" t="n"/>
+      <c r="C58" s="8" t="n"/>
+      <c r="D58" s="8" t="n"/>
+      <c r="E58" s="8" t="n"/>
+      <c r="F58" s="8" t="n"/>
+      <c r="G58" s="8" t="n"/>
+      <c r="H58" s="8" t="n"/>
+      <c r="I58" s="8" t="n"/>
+      <c r="J58" s="8" t="n"/>
+      <c r="K58" s="8" t="n"/>
+      <c r="L58" s="8" t="n"/>
+      <c r="M58" s="8" t="n"/>
+      <c r="N58" s="8" t="n"/>
+      <c r="O58" s="8" t="n"/>
+      <c r="P58" s="8" t="n"/>
+      <c r="Q58" s="8" t="n"/>
+      <c r="R58" s="8" t="n"/>
+      <c r="S58" s="8" t="n"/>
+      <c r="T58" s="8" t="n"/>
+      <c r="U58" s="8" t="n"/>
+      <c r="V58" s="8" t="n"/>
+      <c r="W58" s="8" t="n"/>
+      <c r="X58" s="8" t="n"/>
+      <c r="Y58" s="8" t="n"/>
+      <c r="Z58" s="8" t="n"/>
+      <c r="AA58" s="8" t="n"/>
+      <c r="AB58" s="8" t="n"/>
+      <c r="AC58" s="8" t="n"/>
+      <c r="AD58" s="8" t="n"/>
+      <c r="AE58" s="8" t="n"/>
+      <c r="AF58" s="8" t="n"/>
+      <c r="AG58" s="8" t="n"/>
+      <c r="AH58" s="8" t="n"/>
+      <c r="AI58" s="8" t="n"/>
+      <c r="AJ58" s="8" t="n"/>
+      <c r="AK58" s="8" t="n"/>
+      <c r="AL58" s="8" t="n"/>
+      <c r="AM58" s="8" t="n"/>
+      <c r="AN58" s="8" t="n"/>
+      <c r="AO58" s="8" t="n"/>
+      <c r="AP58" s="8" t="n"/>
+      <c r="AQ58" s="8" t="n"/>
+      <c r="AR58" s="8" t="n"/>
+      <c r="AS58" s="8" t="n"/>
+      <c r="AT58" s="8" t="n"/>
+      <c r="AU58" s="8" t="n"/>
+      <c r="AV58" s="8" t="n"/>
+      <c r="AW58" s="8" t="n"/>
+      <c r="AX58" s="8" t="n"/>
+      <c r="AY58" s="8" t="n"/>
+      <c r="AZ58" s="8" t="n"/>
+      <c r="BA58" s="8" t="n"/>
+      <c r="BB58" s="8" t="n"/>
+      <c r="BC58" s="8" t="n"/>
+      <c r="BD58" s="8" t="n"/>
+      <c r="BE58" s="8" t="n"/>
+      <c r="BF58" s="8" t="n"/>
+      <c r="BG58" s="8" t="n"/>
+      <c r="BH58" s="8" t="n"/>
+      <c r="BI58" s="8" t="n"/>
+      <c r="BJ58" s="8" t="n"/>
+      <c r="BK58" s="8" t="n"/>
+      <c r="BL58" s="8" t="n"/>
+      <c r="BM58" s="8" t="n"/>
+      <c r="BN58" s="8" t="n"/>
+      <c r="BO58" s="8" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="9" t="inlineStr">
         <is>
-          <t>X020</t>
+          <t>L010</t>
         </is>
       </c>
       <c r="B59" s="10" t="inlineStr">
         <is>
-          <t>הכנת תשתית וטיח צבעוני לחזיתות (225 מ״ר)</t>
+          <t>התקנת אלומיניום – חלונות ודלתות חוץ (26 יח׳)</t>
         </is>
       </c>
       <c r="C59" s="10" t="inlineStr">
         <is>
-          <t>14.01</t>
+          <t>16.01</t>
         </is>
       </c>
       <c r="D59" s="9" t="n">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="E59" s="9" t="inlineStr">
         <is>
-          <t>X010</t>
+          <t>A045</t>
         </is>
       </c>
       <c r="F59" s="9" t="inlineStr">
         <is>
-          <t>L010</t>
-        </is>
-      </c>
-      <c r="G59" s="9" t="inlineStr">
-        <is>
-          <t>R020</t>
-        </is>
-      </c>
+          <t>K050</t>
+        </is>
+      </c>
+      <c r="G59" s="9" t="n"/>
       <c r="H59" s="9" t="n"/>
       <c r="I59" s="9" t="n"/>
       <c r="J59" s="9" t="n"/>
       <c r="K59" s="11">
-        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$86,MATCH(E59,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(F59,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(G59,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(H59,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(I59,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(J59,$A$6:$A$86,0)),0))</f>
+        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$88,MATCH(E59,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(F59,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(G59,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(H59,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(I59,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(J59,$A$6:$A$88,0)),0))</f>
         <v/>
       </c>
       <c r="L59" s="11">
@@ -3832,45 +3832,53 @@
       <c r="N59" s="9" t="n"/>
       <c r="O59" s="10" t="inlineStr">
         <is>
-          <t>הנחה: ~12 מ״ר ליום</t>
+          <t>הנחה</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="9" t="inlineStr">
         <is>
-          <t>Z010</t>
+          <t>X020</t>
         </is>
       </c>
       <c r="B60" s="10" t="inlineStr">
         <is>
-          <t>אדני חלונות וספי דלתות ואיטום סביבם</t>
+          <t>הכנת תשתית וטיח צבעוני לחזיתות (225 מ״ר)</t>
         </is>
       </c>
       <c r="C60" s="10" t="inlineStr">
         <is>
-          <t>12.01–12.04</t>
+          <t>14.01</t>
         </is>
       </c>
       <c r="D60" s="9" t="n">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="E60" s="9" t="inlineStr">
         <is>
+          <t>X010</t>
+        </is>
+      </c>
+      <c r="F60" s="9" t="inlineStr">
+        <is>
           <t>L010</t>
         </is>
       </c>
-      <c r="F60" s="9" t="inlineStr">
-        <is>
-          <t>X020</t>
-        </is>
-      </c>
-      <c r="G60" s="9" t="n"/>
-      <c r="H60" s="9" t="n"/>
+      <c r="G60" s="9" t="inlineStr">
+        <is>
+          <t>R020</t>
+        </is>
+      </c>
+      <c r="H60" s="9" t="inlineStr">
+        <is>
+          <t>D070</t>
+        </is>
+      </c>
       <c r="I60" s="9" t="n"/>
       <c r="J60" s="9" t="n"/>
       <c r="K60" s="11">
-        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$86,MATCH(E60,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(F60,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(G60,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(H60,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(I60,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(J60,$A$6:$A$86,0)),0))</f>
+        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$88,MATCH(E60,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(F60,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(G60,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(H60,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(I60,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(J60,$A$6:$A$88,0)),0))</f>
         <v/>
       </c>
       <c r="L60" s="11">
@@ -3884,122 +3892,101 @@
       <c r="N60" s="9" t="n"/>
       <c r="O60" s="10" t="inlineStr">
         <is>
+          <t>הנחה: ~12 מ״ר ליום</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="9" t="inlineStr">
+        <is>
+          <t>Z010</t>
+        </is>
+      </c>
+      <c r="B61" s="10" t="inlineStr">
+        <is>
+          <t>אדני חלונות וספי דלתות ואיטום סביבם</t>
+        </is>
+      </c>
+      <c r="C61" s="10" t="inlineStr">
+        <is>
+          <t>12.01–12.04</t>
+        </is>
+      </c>
+      <c r="D61" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="E61" s="9" t="inlineStr">
+        <is>
+          <t>L010</t>
+        </is>
+      </c>
+      <c r="F61" s="9" t="inlineStr">
+        <is>
+          <t>X020</t>
+        </is>
+      </c>
+      <c r="G61" s="9" t="n"/>
+      <c r="H61" s="9" t="n"/>
+      <c r="I61" s="9" t="n"/>
+      <c r="J61" s="9" t="n"/>
+      <c r="K61" s="11">
+        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$88,MATCH(E61,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(F61,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(G61,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(H61,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(I61,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(J61,$A$6:$A$88,0)),0))</f>
+        <v/>
+      </c>
+      <c r="L61" s="11">
+        <f>IF(D61=0,IF(COUNTA(E61:J61)=0,$D$2,K61),WORKDAY.INTL(K61,1,$D$3))</f>
+        <v/>
+      </c>
+      <c r="M61" s="11">
+        <f>IF(D61=0,L61,WORKDAY.INTL(L61,D61-1,$D$3))</f>
+        <v/>
+      </c>
+      <c r="N61" s="9" t="n"/>
+      <c r="O61" s="10" t="inlineStr">
+        <is>
           <t>הנחה</t>
         </is>
       </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="7" t="inlineStr">
-        <is>
-          <t>8. גמרים פנים</t>
-        </is>
-      </c>
-      <c r="B61" s="8" t="n"/>
-      <c r="C61" s="8" t="n"/>
-      <c r="D61" s="8" t="n"/>
-      <c r="E61" s="8" t="n"/>
-      <c r="F61" s="8" t="n"/>
-      <c r="G61" s="8" t="n"/>
-      <c r="H61" s="8" t="n"/>
-      <c r="I61" s="8" t="n"/>
-      <c r="J61" s="8" t="n"/>
-      <c r="K61" s="8" t="n"/>
-      <c r="L61" s="8" t="n"/>
-      <c r="M61" s="8" t="n"/>
-      <c r="N61" s="8" t="n"/>
-      <c r="O61" s="8" t="n"/>
-      <c r="P61" s="8" t="n"/>
-      <c r="Q61" s="8" t="n"/>
-      <c r="R61" s="8" t="n"/>
-      <c r="S61" s="8" t="n"/>
-      <c r="T61" s="8" t="n"/>
-      <c r="U61" s="8" t="n"/>
-      <c r="V61" s="8" t="n"/>
-      <c r="W61" s="8" t="n"/>
-      <c r="X61" s="8" t="n"/>
-      <c r="Y61" s="8" t="n"/>
-      <c r="Z61" s="8" t="n"/>
-      <c r="AA61" s="8" t="n"/>
-      <c r="AB61" s="8" t="n"/>
-      <c r="AC61" s="8" t="n"/>
-      <c r="AD61" s="8" t="n"/>
-      <c r="AE61" s="8" t="n"/>
-      <c r="AF61" s="8" t="n"/>
-      <c r="AG61" s="8" t="n"/>
-      <c r="AH61" s="8" t="n"/>
-      <c r="AI61" s="8" t="n"/>
-      <c r="AJ61" s="8" t="n"/>
-      <c r="AK61" s="8" t="n"/>
-      <c r="AL61" s="8" t="n"/>
-      <c r="AM61" s="8" t="n"/>
-      <c r="AN61" s="8" t="n"/>
-      <c r="AO61" s="8" t="n"/>
-      <c r="AP61" s="8" t="n"/>
-      <c r="AQ61" s="8" t="n"/>
-      <c r="AR61" s="8" t="n"/>
-      <c r="AS61" s="8" t="n"/>
-      <c r="AT61" s="8" t="n"/>
-      <c r="AU61" s="8" t="n"/>
-      <c r="AV61" s="8" t="n"/>
-      <c r="AW61" s="8" t="n"/>
-      <c r="AX61" s="8" t="n"/>
-      <c r="AY61" s="8" t="n"/>
-      <c r="AZ61" s="8" t="n"/>
-      <c r="BA61" s="8" t="n"/>
-      <c r="BB61" s="8" t="n"/>
-      <c r="BC61" s="8" t="n"/>
-      <c r="BD61" s="8" t="n"/>
-      <c r="BE61" s="8" t="n"/>
-      <c r="BF61" s="8" t="n"/>
-      <c r="BG61" s="8" t="n"/>
-      <c r="BH61" s="8" t="n"/>
-      <c r="BI61" s="8" t="n"/>
-      <c r="BJ61" s="8" t="n"/>
-      <c r="BK61" s="8" t="n"/>
-      <c r="BL61" s="8" t="n"/>
-      <c r="BM61" s="8" t="n"/>
-      <c r="BN61" s="8" t="n"/>
-      <c r="BO61" s="8" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="9" t="inlineStr">
         <is>
-          <t>M020</t>
+          <t>X030</t>
         </is>
       </c>
       <c r="B62" s="10" t="inlineStr">
         <is>
-          <t>התקנת יחידות מיזוג, בדיקות ואקום ולחץ</t>
+          <t>פירוק פיגום חיצוני</t>
         </is>
       </c>
       <c r="C62" s="10" t="inlineStr">
         <is>
-          <t>08.01, 08.03, 08.04</t>
+          <t>01.09</t>
         </is>
       </c>
       <c r="D62" s="9" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="E62" s="9" t="inlineStr">
         <is>
-          <t>G030</t>
+          <t>X020</t>
         </is>
       </c>
       <c r="F62" s="9" t="inlineStr">
         <is>
-          <t>M010</t>
+          <t>R040</t>
         </is>
       </c>
       <c r="G62" s="9" t="inlineStr">
         <is>
-          <t>A065</t>
+          <t>Z010</t>
         </is>
       </c>
       <c r="H62" s="9" t="n"/>
       <c r="I62" s="9" t="n"/>
       <c r="J62" s="9" t="n"/>
       <c r="K62" s="11">
-        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$86,MATCH(E62,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(F62,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(G62,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(H62,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(I62,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(J62,$A$6:$A$86,0)),0))</f>
+        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$88,MATCH(E62,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(F62,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(G62,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(H62,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(I62,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(J62,$A$6:$A$88,0)),0))</f>
         <v/>
       </c>
       <c r="L62" s="11">
@@ -4010,112 +3997,125 @@
         <f>IF(D62=0,L62,WORKDAY.INTL(L62,D62-1,$D$3))</f>
         <v/>
       </c>
-      <c r="N62" s="12" t="inlineStr">
-        <is>
-          <t>כן</t>
-        </is>
-      </c>
+      <c r="N62" s="9" t="n"/>
       <c r="O62" s="10" t="inlineStr">
         <is>
-          <t>הנחה; מפרט: מיזוג נבדק לפני טיח וצבע</t>
+          <t>הנחה</t>
         </is>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="9" t="inlineStr">
-        <is>
-          <t>F010</t>
-        </is>
-      </c>
-      <c r="B63" s="10" t="inlineStr">
-        <is>
-          <t>תיקוני טיח ושפכטל, ידיים ראשונות (576 מ״ר)</t>
-        </is>
-      </c>
-      <c r="C63" s="10" t="inlineStr">
-        <is>
-          <t>15.01–15.03</t>
-        </is>
-      </c>
-      <c r="D63" s="9" t="n">
-        <v>12</v>
-      </c>
-      <c r="E63" s="9" t="inlineStr">
-        <is>
-          <t>G030</t>
-        </is>
-      </c>
-      <c r="F63" s="9" t="inlineStr">
-        <is>
-          <t>M020</t>
-        </is>
-      </c>
-      <c r="G63" s="9" t="n"/>
-      <c r="H63" s="9" t="n"/>
-      <c r="I63" s="9" t="n"/>
-      <c r="J63" s="9" t="n"/>
-      <c r="K63" s="11">
-        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$86,MATCH(E63,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(F63,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(G63,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(H63,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(I63,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(J63,$A$6:$A$86,0)),0))</f>
-        <v/>
-      </c>
-      <c r="L63" s="11">
-        <f>IF(D63=0,IF(COUNTA(E63:J63)=0,$D$2,K63),WORKDAY.INTL(K63,1,$D$3))</f>
-        <v/>
-      </c>
-      <c r="M63" s="11">
-        <f>IF(D63=0,L63,WORKDAY.INTL(L63,D63-1,$D$3))</f>
-        <v/>
-      </c>
-      <c r="N63" s="12" t="inlineStr">
-        <is>
-          <t>כן</t>
-        </is>
-      </c>
-      <c r="O63" s="10" t="inlineStr">
-        <is>
-          <t>הנחה</t>
-        </is>
-      </c>
+      <c r="A63" s="7" t="inlineStr">
+        <is>
+          <t>8. גמרים פנים</t>
+        </is>
+      </c>
+      <c r="B63" s="8" t="n"/>
+      <c r="C63" s="8" t="n"/>
+      <c r="D63" s="8" t="n"/>
+      <c r="E63" s="8" t="n"/>
+      <c r="F63" s="8" t="n"/>
+      <c r="G63" s="8" t="n"/>
+      <c r="H63" s="8" t="n"/>
+      <c r="I63" s="8" t="n"/>
+      <c r="J63" s="8" t="n"/>
+      <c r="K63" s="8" t="n"/>
+      <c r="L63" s="8" t="n"/>
+      <c r="M63" s="8" t="n"/>
+      <c r="N63" s="8" t="n"/>
+      <c r="O63" s="8" t="n"/>
+      <c r="P63" s="8" t="n"/>
+      <c r="Q63" s="8" t="n"/>
+      <c r="R63" s="8" t="n"/>
+      <c r="S63" s="8" t="n"/>
+      <c r="T63" s="8" t="n"/>
+      <c r="U63" s="8" t="n"/>
+      <c r="V63" s="8" t="n"/>
+      <c r="W63" s="8" t="n"/>
+      <c r="X63" s="8" t="n"/>
+      <c r="Y63" s="8" t="n"/>
+      <c r="Z63" s="8" t="n"/>
+      <c r="AA63" s="8" t="n"/>
+      <c r="AB63" s="8" t="n"/>
+      <c r="AC63" s="8" t="n"/>
+      <c r="AD63" s="8" t="n"/>
+      <c r="AE63" s="8" t="n"/>
+      <c r="AF63" s="8" t="n"/>
+      <c r="AG63" s="8" t="n"/>
+      <c r="AH63" s="8" t="n"/>
+      <c r="AI63" s="8" t="n"/>
+      <c r="AJ63" s="8" t="n"/>
+      <c r="AK63" s="8" t="n"/>
+      <c r="AL63" s="8" t="n"/>
+      <c r="AM63" s="8" t="n"/>
+      <c r="AN63" s="8" t="n"/>
+      <c r="AO63" s="8" t="n"/>
+      <c r="AP63" s="8" t="n"/>
+      <c r="AQ63" s="8" t="n"/>
+      <c r="AR63" s="8" t="n"/>
+      <c r="AS63" s="8" t="n"/>
+      <c r="AT63" s="8" t="n"/>
+      <c r="AU63" s="8" t="n"/>
+      <c r="AV63" s="8" t="n"/>
+      <c r="AW63" s="8" t="n"/>
+      <c r="AX63" s="8" t="n"/>
+      <c r="AY63" s="8" t="n"/>
+      <c r="AZ63" s="8" t="n"/>
+      <c r="BA63" s="8" t="n"/>
+      <c r="BB63" s="8" t="n"/>
+      <c r="BC63" s="8" t="n"/>
+      <c r="BD63" s="8" t="n"/>
+      <c r="BE63" s="8" t="n"/>
+      <c r="BF63" s="8" t="n"/>
+      <c r="BG63" s="8" t="n"/>
+      <c r="BH63" s="8" t="n"/>
+      <c r="BI63" s="8" t="n"/>
+      <c r="BJ63" s="8" t="n"/>
+      <c r="BK63" s="8" t="n"/>
+      <c r="BL63" s="8" t="n"/>
+      <c r="BM63" s="8" t="n"/>
+      <c r="BN63" s="8" t="n"/>
+      <c r="BO63" s="8" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="9" t="inlineStr">
         <is>
-          <t>T010</t>
+          <t>M020</t>
         </is>
       </c>
       <c r="B64" s="10" t="inlineStr">
         <is>
-          <t>ריצוף פנים 120×120 (219.9 מ״ר) ו-120×60 מרתף (105 מ״ר)</t>
+          <t>התקנת יחידות מיזוג, בדיקות ואקום ולחץ</t>
         </is>
       </c>
       <c r="C64" s="10" t="inlineStr">
         <is>
-          <t>13.01, 13.02</t>
+          <t>08.01, 08.03, 08.04</t>
         </is>
       </c>
       <c r="D64" s="9" t="n">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="E64" s="9" t="inlineStr">
         <is>
-          <t>W040</t>
+          <t>G030</t>
         </is>
       </c>
       <c r="F64" s="9" t="inlineStr">
         <is>
-          <t>G030</t>
+          <t>M010</t>
         </is>
       </c>
       <c r="G64" s="9" t="inlineStr">
         <is>
-          <t>A055</t>
+          <t>A065</t>
         </is>
       </c>
       <c r="H64" s="9" t="n"/>
       <c r="I64" s="9" t="n"/>
       <c r="J64" s="9" t="n"/>
       <c r="K64" s="11">
-        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$86,MATCH(E64,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(F64,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(G64,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(H64,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(I64,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(J64,$A$6:$A$86,0)),0))</f>
+        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$88,MATCH(E64,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(F64,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(G64,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(H64,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(I64,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(J64,$A$6:$A$88,0)),0))</f>
         <v/>
       </c>
       <c r="L64" s="11">
@@ -4126,40 +4126,44 @@
         <f>IF(D64=0,L64,WORKDAY.INTL(L64,D64-1,$D$3))</f>
         <v/>
       </c>
-      <c r="N64" s="9" t="n"/>
+      <c r="N64" s="12" t="inlineStr">
+        <is>
+          <t>כן</t>
+        </is>
+      </c>
       <c r="O64" s="10" t="inlineStr">
         <is>
-          <t>הנחה: ~25 מ״ר ליום</t>
+          <t>הנחה; מפרט: מיזוג נבדק לפני טיח וצבע</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="9" t="inlineStr">
         <is>
-          <t>T020</t>
+          <t>F010</t>
         </is>
       </c>
       <c r="B65" s="10" t="inlineStr">
         <is>
-          <t>חיפוי קירות מקלחות (121.2 מ״ר)</t>
+          <t>תיקוני טיח ושפכטל, ידיים ראשונות (576 מ״ר)</t>
         </is>
       </c>
       <c r="C65" s="10" t="inlineStr">
         <is>
-          <t>13.03</t>
+          <t>15.01–15.03</t>
         </is>
       </c>
       <c r="D65" s="9" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="E65" s="9" t="inlineStr">
         <is>
-          <t>W040</t>
+          <t>G030</t>
         </is>
       </c>
       <c r="F65" s="9" t="inlineStr">
         <is>
-          <t>A055</t>
+          <t>M020</t>
         </is>
       </c>
       <c r="G65" s="9" t="n"/>
@@ -4167,7 +4171,7 @@
       <c r="I65" s="9" t="n"/>
       <c r="J65" s="9" t="n"/>
       <c r="K65" s="11">
-        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$86,MATCH(E65,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(F65,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(G65,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(H65,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(I65,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(J65,$A$6:$A$86,0)),0))</f>
+        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$88,MATCH(E65,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(F65,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(G65,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(H65,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(I65,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(J65,$A$6:$A$88,0)),0))</f>
         <v/>
       </c>
       <c r="L65" s="11">
@@ -4178,7 +4182,11 @@
         <f>IF(D65=0,L65,WORKDAY.INTL(L65,D65-1,$D$3))</f>
         <v/>
       </c>
-      <c r="N65" s="9" t="n"/>
+      <c r="N65" s="12" t="inlineStr">
+        <is>
+          <t>כן</t>
+        </is>
+      </c>
       <c r="O65" s="10" t="inlineStr">
         <is>
           <t>הנחה</t>
@@ -4188,17 +4196,17 @@
     <row r="66">
       <c r="A66" s="9" t="inlineStr">
         <is>
-          <t>T030</t>
+          <t>T010</t>
         </is>
       </c>
       <c r="B66" s="10" t="inlineStr">
         <is>
-          <t>ריצוף חוץ ומרפסות R11 (263.7 מ״ר)</t>
+          <t>ריצוף פנים 120×120 (219.9 מ״ר) ו-120×60 מרתף (105 מ״ר)</t>
         </is>
       </c>
       <c r="C66" s="10" t="inlineStr">
         <is>
-          <t>13.05</t>
+          <t>13.01, 13.02</t>
         </is>
       </c>
       <c r="D66" s="9" t="n">
@@ -4206,20 +4214,24 @@
       </c>
       <c r="E66" s="9" t="inlineStr">
         <is>
-          <t>W030</t>
+          <t>W040</t>
         </is>
       </c>
       <c r="F66" s="9" t="inlineStr">
         <is>
+          <t>G030</t>
+        </is>
+      </c>
+      <c r="G66" s="9" t="inlineStr">
+        <is>
           <t>A055</t>
         </is>
       </c>
-      <c r="G66" s="9" t="n"/>
       <c r="H66" s="9" t="n"/>
       <c r="I66" s="9" t="n"/>
       <c r="J66" s="9" t="n"/>
       <c r="K66" s="11">
-        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$86,MATCH(E66,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(F66,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(G66,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(H66,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(I66,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(J66,$A$6:$A$86,0)),0))</f>
+        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$88,MATCH(E66,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(F66,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(G66,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(H66,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(I66,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(J66,$A$6:$A$88,0)),0))</f>
         <v/>
       </c>
       <c r="L66" s="11">
@@ -4233,24 +4245,24 @@
       <c r="N66" s="9" t="n"/>
       <c r="O66" s="10" t="inlineStr">
         <is>
-          <t>הנחה</t>
+          <t>הנחה: ~25 מ״ר ליום</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="9" t="inlineStr">
         <is>
-          <t>T040</t>
+          <t>T020</t>
         </is>
       </c>
       <c r="B67" s="10" t="inlineStr">
         <is>
-          <t>חיפוי מדרגות פנים (50 מ״א) והתקנת פנלים (285 מ״א)</t>
+          <t>חיפוי קירות מקלחות (121.2 מ״ר)</t>
         </is>
       </c>
       <c r="C67" s="10" t="inlineStr">
         <is>
-          <t>13.04, 13.07</t>
+          <t>13.03</t>
         </is>
       </c>
       <c r="D67" s="9" t="n">
@@ -4258,12 +4270,12 @@
       </c>
       <c r="E67" s="9" t="inlineStr">
         <is>
-          <t>T010</t>
+          <t>W040</t>
         </is>
       </c>
       <c r="F67" s="9" t="inlineStr">
         <is>
-          <t>K050</t>
+          <t>A055</t>
         </is>
       </c>
       <c r="G67" s="9" t="n"/>
@@ -4271,7 +4283,7 @@
       <c r="I67" s="9" t="n"/>
       <c r="J67" s="9" t="n"/>
       <c r="K67" s="11">
-        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$86,MATCH(E67,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(F67,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(G67,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(H67,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(I67,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(J67,$A$6:$A$86,0)),0))</f>
+        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$88,MATCH(E67,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(F67,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(G67,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(H67,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(I67,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(J67,$A$6:$A$88,0)),0))</f>
         <v/>
       </c>
       <c r="L67" s="11">
@@ -4292,30 +4304,30 @@
     <row r="68">
       <c r="A68" s="9" t="inlineStr">
         <is>
-          <t>E030</t>
+          <t>T030</t>
         </is>
       </c>
       <c r="B68" s="10" t="inlineStr">
         <is>
-          <t>התקנת גופי תאורה, ספוטים ומאווררים</t>
+          <t>ריצוף חוץ ומרפסות R11 (263.7 מ״ר)</t>
         </is>
       </c>
       <c r="C68" s="10" t="inlineStr">
         <is>
-          <t>07.03–07.19</t>
+          <t>13.05</t>
         </is>
       </c>
       <c r="D68" s="9" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E68" s="9" t="inlineStr">
         <is>
-          <t>F010</t>
+          <t>W030</t>
         </is>
       </c>
       <c r="F68" s="9" t="inlineStr">
         <is>
-          <t>T010</t>
+          <t>A055</t>
         </is>
       </c>
       <c r="G68" s="9" t="n"/>
@@ -4323,7 +4335,7 @@
       <c r="I68" s="9" t="n"/>
       <c r="J68" s="9" t="n"/>
       <c r="K68" s="11">
-        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$86,MATCH(E68,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(F68,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(G68,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(H68,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(I68,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(J68,$A$6:$A$86,0)),0))</f>
+        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$88,MATCH(E68,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(F68,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(G68,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(H68,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(I68,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(J68,$A$6:$A$88,0)),0))</f>
         <v/>
       </c>
       <c r="L68" s="11">
@@ -4334,60 +4346,48 @@
         <f>IF(D68=0,L68,WORKDAY.INTL(L68,D68-1,$D$3))</f>
         <v/>
       </c>
-      <c r="N68" s="12" t="inlineStr">
-        <is>
-          <t>כן</t>
-        </is>
-      </c>
+      <c r="N68" s="9" t="n"/>
       <c r="O68" s="10" t="inlineStr">
         <is>
-          <t>הנחה; מפרט: לפני הצבע הסופי</t>
+          <t>הנחה</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="9" t="inlineStr">
         <is>
-          <t>F020</t>
+          <t>T040</t>
         </is>
       </c>
       <c r="B69" s="10" t="inlineStr">
         <is>
-          <t>צבע פנים – ידיים סופיות</t>
+          <t>חיפוי מדרגות פנים (50 מ״א) והתקנת פנלים (285 מ״א)</t>
         </is>
       </c>
       <c r="C69" s="10" t="inlineStr">
         <is>
-          <t>15.01–15.03</t>
+          <t>13.04, 13.07</t>
         </is>
       </c>
       <c r="D69" s="9" t="n">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="E69" s="9" t="inlineStr">
         <is>
-          <t>E030</t>
+          <t>T010</t>
         </is>
       </c>
       <c r="F69" s="9" t="inlineStr">
         <is>
-          <t>T020</t>
-        </is>
-      </c>
-      <c r="G69" s="9" t="inlineStr">
-        <is>
-          <t>T040</t>
-        </is>
-      </c>
-      <c r="H69" s="9" t="inlineStr">
-        <is>
-          <t>F010</t>
-        </is>
-      </c>
+          <t>K050</t>
+        </is>
+      </c>
+      <c r="G69" s="9" t="n"/>
+      <c r="H69" s="9" t="n"/>
       <c r="I69" s="9" t="n"/>
       <c r="J69" s="9" t="n"/>
       <c r="K69" s="11">
-        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$86,MATCH(E69,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(F69,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(G69,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(H69,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(I69,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(J69,$A$6:$A$86,0)),0))</f>
+        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$88,MATCH(E69,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(F69,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(G69,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(H69,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(I69,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(J69,$A$6:$A$88,0)),0))</f>
         <v/>
       </c>
       <c r="L69" s="11">
@@ -4398,11 +4398,7 @@
         <f>IF(D69=0,L69,WORKDAY.INTL(L69,D69-1,$D$3))</f>
         <v/>
       </c>
-      <c r="N69" s="12" t="inlineStr">
-        <is>
-          <t>כן</t>
-        </is>
-      </c>
+      <c r="N69" s="9" t="n"/>
       <c r="O69" s="10" t="inlineStr">
         <is>
           <t>הנחה</t>
@@ -4412,34 +4408,38 @@
     <row r="70">
       <c r="A70" s="9" t="inlineStr">
         <is>
-          <t>E020</t>
+          <t>E030</t>
         </is>
       </c>
       <c r="B70" s="10" t="inlineStr">
         <is>
-          <t>התקנת שקעים, מפסקים ואביזרים</t>
+          <t>התקנת גופי תאורה, ספוטים ומאווררים</t>
         </is>
       </c>
       <c r="C70" s="10" t="inlineStr">
         <is>
-          <t>06.01–06.05, 06.10</t>
+          <t>07.03–07.19</t>
         </is>
       </c>
       <c r="D70" s="9" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="E70" s="9" t="inlineStr">
         <is>
-          <t>F020</t>
-        </is>
-      </c>
-      <c r="F70" s="9" t="n"/>
+          <t>F010</t>
+        </is>
+      </c>
+      <c r="F70" s="9" t="inlineStr">
+        <is>
+          <t>T010</t>
+        </is>
+      </c>
       <c r="G70" s="9" t="n"/>
       <c r="H70" s="9" t="n"/>
       <c r="I70" s="9" t="n"/>
       <c r="J70" s="9" t="n"/>
       <c r="K70" s="11">
-        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$86,MATCH(E70,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(F70,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(G70,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(H70,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(I70,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(J70,$A$6:$A$86,0)),0))</f>
+        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$88,MATCH(E70,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(F70,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(G70,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(H70,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(I70,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(J70,$A$6:$A$88,0)),0))</f>
         <v/>
       </c>
       <c r="L70" s="11">
@@ -4450,35 +4450,39 @@
         <f>IF(D70=0,L70,WORKDAY.INTL(L70,D70-1,$D$3))</f>
         <v/>
       </c>
-      <c r="N70" s="9" t="n"/>
+      <c r="N70" s="12" t="inlineStr">
+        <is>
+          <t>כן</t>
+        </is>
+      </c>
       <c r="O70" s="10" t="inlineStr">
         <is>
-          <t>הנחה</t>
+          <t>הנחה; מפרט: לפני הצבע הסופי</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="9" t="inlineStr">
         <is>
-          <t>P020</t>
+          <t>F020</t>
         </is>
       </c>
       <c r="B71" s="10" t="inlineStr">
         <is>
-          <t>התקנת כלים סניטריים, ברזים ודוד</t>
+          <t>צבע פנים – ידיים סופיות</t>
         </is>
       </c>
       <c r="C71" s="10" t="inlineStr">
         <is>
-          <t>05.01–05.24, 05.34</t>
+          <t>15.01–15.03</t>
         </is>
       </c>
       <c r="D71" s="9" t="n">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="E71" s="9" t="inlineStr">
         <is>
-          <t>F020</t>
+          <t>E030</t>
         </is>
       </c>
       <c r="F71" s="9" t="inlineStr">
@@ -4486,12 +4490,20 @@
           <t>T020</t>
         </is>
       </c>
-      <c r="G71" s="9" t="n"/>
-      <c r="H71" s="9" t="n"/>
+      <c r="G71" s="9" t="inlineStr">
+        <is>
+          <t>T040</t>
+        </is>
+      </c>
+      <c r="H71" s="9" t="inlineStr">
+        <is>
+          <t>F010</t>
+        </is>
+      </c>
       <c r="I71" s="9" t="n"/>
       <c r="J71" s="9" t="n"/>
       <c r="K71" s="11">
-        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$86,MATCH(E71,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(F71,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(G71,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(H71,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(I71,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(J71,$A$6:$A$86,0)),0))</f>
+        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$88,MATCH(E71,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(F71,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(G71,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(H71,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(I71,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(J71,$A$6:$A$88,0)),0))</f>
         <v/>
       </c>
       <c r="L71" s="11">
@@ -4516,38 +4528,34 @@
     <row r="72">
       <c r="A72" s="9" t="inlineStr">
         <is>
-          <t>L020</t>
+          <t>E020</t>
         </is>
       </c>
       <c r="B72" s="10" t="inlineStr">
         <is>
-          <t>דלתות פנים וכניסה (14 יח׳)</t>
+          <t>התקנת שקעים, מפסקים ואביזרים</t>
         </is>
       </c>
       <c r="C72" s="10" t="inlineStr">
         <is>
-          <t>16.02–16.04</t>
+          <t>06.01–06.05, 06.10</t>
         </is>
       </c>
       <c r="D72" s="9" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E72" s="9" t="inlineStr">
         <is>
           <t>F020</t>
         </is>
       </c>
-      <c r="F72" s="9" t="inlineStr">
-        <is>
-          <t>A045</t>
-        </is>
-      </c>
+      <c r="F72" s="9" t="n"/>
       <c r="G72" s="9" t="n"/>
       <c r="H72" s="9" t="n"/>
       <c r="I72" s="9" t="n"/>
       <c r="J72" s="9" t="n"/>
       <c r="K72" s="11">
-        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$86,MATCH(E72,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(F72,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(G72,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(H72,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(I72,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(J72,$A$6:$A$86,0)),0))</f>
+        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$88,MATCH(E72,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(F72,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(G72,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(H72,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(I72,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(J72,$A$6:$A$88,0)),0))</f>
         <v/>
       </c>
       <c r="L72" s="11">
@@ -4568,17 +4576,17 @@
     <row r="73">
       <c r="A73" s="9" t="inlineStr">
         <is>
-          <t>L030</t>
+          <t>P020</t>
         </is>
       </c>
       <c r="B73" s="10" t="inlineStr">
         <is>
-          <t>שערים חשמליים ואינטרקום שער</t>
+          <t>התקנת כלים סניטריים, ברזים ודוד</t>
         </is>
       </c>
       <c r="C73" s="10" t="inlineStr">
         <is>
-          <t>16.05–16.07, 18.03</t>
+          <t>05.01–05.24, 05.34</t>
         </is>
       </c>
       <c r="D73" s="9" t="n">
@@ -4586,12 +4594,12 @@
       </c>
       <c r="E73" s="9" t="inlineStr">
         <is>
-          <t>A060</t>
+          <t>F020</t>
         </is>
       </c>
       <c r="F73" s="9" t="inlineStr">
         <is>
-          <t>X020</t>
+          <t>T020</t>
         </is>
       </c>
       <c r="G73" s="9" t="n"/>
@@ -4599,7 +4607,7 @@
       <c r="I73" s="9" t="n"/>
       <c r="J73" s="9" t="n"/>
       <c r="K73" s="11">
-        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$86,MATCH(E73,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(F73,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(G73,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(H73,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(I73,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(J73,$A$6:$A$86,0)),0))</f>
+        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$88,MATCH(E73,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(F73,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(G73,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(H73,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(I73,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(J73,$A$6:$A$88,0)),0))</f>
         <v/>
       </c>
       <c r="L73" s="11">
@@ -4610,7 +4618,11 @@
         <f>IF(D73=0,L73,WORKDAY.INTL(L73,D73-1,$D$3))</f>
         <v/>
       </c>
-      <c r="N73" s="9" t="n"/>
+      <c r="N73" s="12" t="inlineStr">
+        <is>
+          <t>כן</t>
+        </is>
+      </c>
       <c r="O73" s="10" t="inlineStr">
         <is>
           <t>הנחה</t>
@@ -4620,30 +4632,30 @@
     <row r="74">
       <c r="A74" s="9" t="inlineStr">
         <is>
-          <t>L040</t>
+          <t>L020</t>
         </is>
       </c>
       <c r="B74" s="10" t="inlineStr">
         <is>
-          <t>תריסים חשמליים (18 יח׳)</t>
+          <t>דלתות פנים וכניסה (14 יח׳)</t>
         </is>
       </c>
       <c r="C74" s="10" t="inlineStr">
         <is>
-          <t>16.09</t>
+          <t>16.02–16.04</t>
         </is>
       </c>
       <c r="D74" s="9" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E74" s="9" t="inlineStr">
         <is>
-          <t>A060</t>
+          <t>F020</t>
         </is>
       </c>
       <c r="F74" s="9" t="inlineStr">
         <is>
-          <t>L010</t>
+          <t>A045</t>
         </is>
       </c>
       <c r="G74" s="9" t="n"/>
@@ -4651,7 +4663,7 @@
       <c r="I74" s="9" t="n"/>
       <c r="J74" s="9" t="n"/>
       <c r="K74" s="11">
-        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$86,MATCH(E74,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(F74,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(G74,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(H74,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(I74,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(J74,$A$6:$A$86,0)),0))</f>
+        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$88,MATCH(E74,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(F74,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(G74,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(H74,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(I74,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(J74,$A$6:$A$88,0)),0))</f>
         <v/>
       </c>
       <c r="L74" s="11">
@@ -4665,41 +4677,45 @@
       <c r="N74" s="9" t="n"/>
       <c r="O74" s="10" t="inlineStr">
         <is>
-          <t>הנחה; אופציה</t>
+          <t>הנחה</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="9" t="inlineStr">
         <is>
-          <t>C020</t>
+          <t>L030</t>
         </is>
       </c>
       <c r="B75" s="10" t="inlineStr">
         <is>
-          <t>נקודות תקשורת, לוח תקשורת ובדיקות רציפות</t>
+          <t>שערים חשמליים ואינטרקום שער</t>
         </is>
       </c>
       <c r="C75" s="10" t="inlineStr">
         <is>
-          <t>18.02, 18.04, 18.05</t>
+          <t>16.05–16.07, 18.03</t>
         </is>
       </c>
       <c r="D75" s="9" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E75" s="9" t="inlineStr">
         <is>
-          <t>F020</t>
-        </is>
-      </c>
-      <c r="F75" s="9" t="n"/>
+          <t>A060</t>
+        </is>
+      </c>
+      <c r="F75" s="9" t="inlineStr">
+        <is>
+          <t>X020</t>
+        </is>
+      </c>
       <c r="G75" s="9" t="n"/>
       <c r="H75" s="9" t="n"/>
       <c r="I75" s="9" t="n"/>
       <c r="J75" s="9" t="n"/>
       <c r="K75" s="11">
-        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$86,MATCH(E75,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(F75,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(G75,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(H75,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(I75,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(J75,$A$6:$A$86,0)),0))</f>
+        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$88,MATCH(E75,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(F75,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(G75,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(H75,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(I75,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(J75,$A$6:$A$88,0)),0))</f>
         <v/>
       </c>
       <c r="L75" s="11">
@@ -4718,113 +4734,88 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="7" t="inlineStr">
-        <is>
-          <t>9. פיתוח וחשמל חוץ</t>
-        </is>
-      </c>
-      <c r="B76" s="8" t="n"/>
-      <c r="C76" s="8" t="n"/>
-      <c r="D76" s="8" t="n"/>
-      <c r="E76" s="8" t="n"/>
-      <c r="F76" s="8" t="n"/>
-      <c r="G76" s="8" t="n"/>
-      <c r="H76" s="8" t="n"/>
-      <c r="I76" s="8" t="n"/>
-      <c r="J76" s="8" t="n"/>
-      <c r="K76" s="8" t="n"/>
-      <c r="L76" s="8" t="n"/>
-      <c r="M76" s="8" t="n"/>
-      <c r="N76" s="8" t="n"/>
-      <c r="O76" s="8" t="n"/>
-      <c r="P76" s="8" t="n"/>
-      <c r="Q76" s="8" t="n"/>
-      <c r="R76" s="8" t="n"/>
-      <c r="S76" s="8" t="n"/>
-      <c r="T76" s="8" t="n"/>
-      <c r="U76" s="8" t="n"/>
-      <c r="V76" s="8" t="n"/>
-      <c r="W76" s="8" t="n"/>
-      <c r="X76" s="8" t="n"/>
-      <c r="Y76" s="8" t="n"/>
-      <c r="Z76" s="8" t="n"/>
-      <c r="AA76" s="8" t="n"/>
-      <c r="AB76" s="8" t="n"/>
-      <c r="AC76" s="8" t="n"/>
-      <c r="AD76" s="8" t="n"/>
-      <c r="AE76" s="8" t="n"/>
-      <c r="AF76" s="8" t="n"/>
-      <c r="AG76" s="8" t="n"/>
-      <c r="AH76" s="8" t="n"/>
-      <c r="AI76" s="8" t="n"/>
-      <c r="AJ76" s="8" t="n"/>
-      <c r="AK76" s="8" t="n"/>
-      <c r="AL76" s="8" t="n"/>
-      <c r="AM76" s="8" t="n"/>
-      <c r="AN76" s="8" t="n"/>
-      <c r="AO76" s="8" t="n"/>
-      <c r="AP76" s="8" t="n"/>
-      <c r="AQ76" s="8" t="n"/>
-      <c r="AR76" s="8" t="n"/>
-      <c r="AS76" s="8" t="n"/>
-      <c r="AT76" s="8" t="n"/>
-      <c r="AU76" s="8" t="n"/>
-      <c r="AV76" s="8" t="n"/>
-      <c r="AW76" s="8" t="n"/>
-      <c r="AX76" s="8" t="n"/>
-      <c r="AY76" s="8" t="n"/>
-      <c r="AZ76" s="8" t="n"/>
-      <c r="BA76" s="8" t="n"/>
-      <c r="BB76" s="8" t="n"/>
-      <c r="BC76" s="8" t="n"/>
-      <c r="BD76" s="8" t="n"/>
-      <c r="BE76" s="8" t="n"/>
-      <c r="BF76" s="8" t="n"/>
-      <c r="BG76" s="8" t="n"/>
-      <c r="BH76" s="8" t="n"/>
-      <c r="BI76" s="8" t="n"/>
-      <c r="BJ76" s="8" t="n"/>
-      <c r="BK76" s="8" t="n"/>
-      <c r="BL76" s="8" t="n"/>
-      <c r="BM76" s="8" t="n"/>
-      <c r="BN76" s="8" t="n"/>
-      <c r="BO76" s="8" t="n"/>
+      <c r="A76" s="9" t="inlineStr">
+        <is>
+          <t>L040</t>
+        </is>
+      </c>
+      <c r="B76" s="10" t="inlineStr">
+        <is>
+          <t>תריסים חשמליים (18 יח׳)</t>
+        </is>
+      </c>
+      <c r="C76" s="10" t="inlineStr">
+        <is>
+          <t>16.09</t>
+        </is>
+      </c>
+      <c r="D76" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="E76" s="9" t="inlineStr">
+        <is>
+          <t>A060</t>
+        </is>
+      </c>
+      <c r="F76" s="9" t="inlineStr">
+        <is>
+          <t>L010</t>
+        </is>
+      </c>
+      <c r="G76" s="9" t="n"/>
+      <c r="H76" s="9" t="n"/>
+      <c r="I76" s="9" t="n"/>
+      <c r="J76" s="9" t="n"/>
+      <c r="K76" s="11">
+        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$88,MATCH(E76,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(F76,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(G76,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(H76,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(I76,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(J76,$A$6:$A$88,0)),0))</f>
+        <v/>
+      </c>
+      <c r="L76" s="11">
+        <f>IF(D76=0,IF(COUNTA(E76:J76)=0,$D$2,K76),WORKDAY.INTL(K76,1,$D$3))</f>
+        <v/>
+      </c>
+      <c r="M76" s="11">
+        <f>IF(D76=0,L76,WORKDAY.INTL(L76,D76-1,$D$3))</f>
+        <v/>
+      </c>
+      <c r="N76" s="9" t="n"/>
+      <c r="O76" s="10" t="inlineStr">
+        <is>
+          <t>הנחה; אופציה</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="9" t="inlineStr">
         <is>
-          <t>E040</t>
+          <t>C020</t>
         </is>
       </c>
       <c r="B77" s="10" t="inlineStr">
         <is>
-          <t>התקנת פילר חברת החשמל והגדלת חיבור</t>
+          <t>נקודות תקשורת, לוח תקשורת ובדיקות רציפות</t>
         </is>
       </c>
       <c r="C77" s="10" t="inlineStr">
         <is>
-          <t>06.07, 06.08</t>
+          <t>18.02, 18.04, 18.05</t>
         </is>
       </c>
       <c r="D77" s="9" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E77" s="9" t="inlineStr">
         <is>
-          <t>A020</t>
-        </is>
-      </c>
-      <c r="F77" s="9" t="inlineStr">
-        <is>
-          <t>S030</t>
-        </is>
-      </c>
+          <t>F020</t>
+        </is>
+      </c>
+      <c r="F77" s="9" t="n"/>
       <c r="G77" s="9" t="n"/>
       <c r="H77" s="9" t="n"/>
       <c r="I77" s="9" t="n"/>
       <c r="J77" s="9" t="n"/>
       <c r="K77" s="11">
-        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$86,MATCH(E77,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(F77,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(G77,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(H77,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(I77,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(J77,$A$6:$A$86,0)),0))</f>
+        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$88,MATCH(E77,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(F77,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(G77,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(H77,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(I77,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(J77,$A$6:$A$88,0)),0))</f>
         <v/>
       </c>
       <c r="L77" s="11">
@@ -4843,80 +4834,105 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="9" t="inlineStr">
-        <is>
-          <t>V010</t>
-        </is>
-      </c>
-      <c r="B78" s="10" t="inlineStr">
-        <is>
-          <t>עבודות עפר ופילוס (65 מ״ר) ומערכת ניקוז מי נגר</t>
-        </is>
-      </c>
-      <c r="C78" s="10" t="inlineStr">
-        <is>
-          <t>17.01, 17.02</t>
-        </is>
-      </c>
-      <c r="D78" s="9" t="n">
-        <v>8</v>
-      </c>
-      <c r="E78" s="9" t="inlineStr">
-        <is>
-          <t>X020</t>
-        </is>
-      </c>
-      <c r="F78" s="9" t="n"/>
-      <c r="G78" s="9" t="n"/>
-      <c r="H78" s="9" t="n"/>
-      <c r="I78" s="9" t="n"/>
-      <c r="J78" s="9" t="n"/>
-      <c r="K78" s="11">
-        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$86,MATCH(E78,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(F78,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(G78,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(H78,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(I78,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(J78,$A$6:$A$86,0)),0))</f>
-        <v/>
-      </c>
-      <c r="L78" s="11">
-        <f>IF(D78=0,IF(COUNTA(E78:J78)=0,$D$2,K78),WORKDAY.INTL(K78,1,$D$3))</f>
-        <v/>
-      </c>
-      <c r="M78" s="11">
-        <f>IF(D78=0,L78,WORKDAY.INTL(L78,D78-1,$D$3))</f>
-        <v/>
-      </c>
-      <c r="N78" s="9" t="n"/>
-      <c r="O78" s="10" t="inlineStr">
-        <is>
-          <t>הנחה</t>
-        </is>
-      </c>
+      <c r="A78" s="7" t="inlineStr">
+        <is>
+          <t>9. פיתוח וחשמל חוץ</t>
+        </is>
+      </c>
+      <c r="B78" s="8" t="n"/>
+      <c r="C78" s="8" t="n"/>
+      <c r="D78" s="8" t="n"/>
+      <c r="E78" s="8" t="n"/>
+      <c r="F78" s="8" t="n"/>
+      <c r="G78" s="8" t="n"/>
+      <c r="H78" s="8" t="n"/>
+      <c r="I78" s="8" t="n"/>
+      <c r="J78" s="8" t="n"/>
+      <c r="K78" s="8" t="n"/>
+      <c r="L78" s="8" t="n"/>
+      <c r="M78" s="8" t="n"/>
+      <c r="N78" s="8" t="n"/>
+      <c r="O78" s="8" t="n"/>
+      <c r="P78" s="8" t="n"/>
+      <c r="Q78" s="8" t="n"/>
+      <c r="R78" s="8" t="n"/>
+      <c r="S78" s="8" t="n"/>
+      <c r="T78" s="8" t="n"/>
+      <c r="U78" s="8" t="n"/>
+      <c r="V78" s="8" t="n"/>
+      <c r="W78" s="8" t="n"/>
+      <c r="X78" s="8" t="n"/>
+      <c r="Y78" s="8" t="n"/>
+      <c r="Z78" s="8" t="n"/>
+      <c r="AA78" s="8" t="n"/>
+      <c r="AB78" s="8" t="n"/>
+      <c r="AC78" s="8" t="n"/>
+      <c r="AD78" s="8" t="n"/>
+      <c r="AE78" s="8" t="n"/>
+      <c r="AF78" s="8" t="n"/>
+      <c r="AG78" s="8" t="n"/>
+      <c r="AH78" s="8" t="n"/>
+      <c r="AI78" s="8" t="n"/>
+      <c r="AJ78" s="8" t="n"/>
+      <c r="AK78" s="8" t="n"/>
+      <c r="AL78" s="8" t="n"/>
+      <c r="AM78" s="8" t="n"/>
+      <c r="AN78" s="8" t="n"/>
+      <c r="AO78" s="8" t="n"/>
+      <c r="AP78" s="8" t="n"/>
+      <c r="AQ78" s="8" t="n"/>
+      <c r="AR78" s="8" t="n"/>
+      <c r="AS78" s="8" t="n"/>
+      <c r="AT78" s="8" t="n"/>
+      <c r="AU78" s="8" t="n"/>
+      <c r="AV78" s="8" t="n"/>
+      <c r="AW78" s="8" t="n"/>
+      <c r="AX78" s="8" t="n"/>
+      <c r="AY78" s="8" t="n"/>
+      <c r="AZ78" s="8" t="n"/>
+      <c r="BA78" s="8" t="n"/>
+      <c r="BB78" s="8" t="n"/>
+      <c r="BC78" s="8" t="n"/>
+      <c r="BD78" s="8" t="n"/>
+      <c r="BE78" s="8" t="n"/>
+      <c r="BF78" s="8" t="n"/>
+      <c r="BG78" s="8" t="n"/>
+      <c r="BH78" s="8" t="n"/>
+      <c r="BI78" s="8" t="n"/>
+      <c r="BJ78" s="8" t="n"/>
+      <c r="BK78" s="8" t="n"/>
+      <c r="BL78" s="8" t="n"/>
+      <c r="BM78" s="8" t="n"/>
+      <c r="BN78" s="8" t="n"/>
+      <c r="BO78" s="8" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="9" t="inlineStr">
         <is>
-          <t>V020</t>
+          <t>E040</t>
         </is>
       </c>
       <c r="B79" s="10" t="inlineStr">
         <is>
-          <t>גינון, השקיה, ברזי גינה ותאורת גן</t>
+          <t>התקנת פילר חברת החשמל והגדלת חיבור</t>
         </is>
       </c>
       <c r="C79" s="10" t="inlineStr">
         <is>
-          <t>17.04, 17.05</t>
+          <t>06.07, 06.08</t>
         </is>
       </c>
       <c r="D79" s="9" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E79" s="9" t="inlineStr">
         <is>
-          <t>V010</t>
+          <t>A020</t>
         </is>
       </c>
       <c r="F79" s="9" t="inlineStr">
         <is>
-          <t>T030</t>
+          <t>S030</t>
         </is>
       </c>
       <c r="G79" s="9" t="n"/>
@@ -4924,7 +4940,7 @@
       <c r="I79" s="9" t="n"/>
       <c r="J79" s="9" t="n"/>
       <c r="K79" s="11">
-        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$86,MATCH(E79,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(F79,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(G79,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(H79,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(I79,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(J79,$A$6:$A$86,0)),0))</f>
+        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$88,MATCH(E79,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(F79,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(G79,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(H79,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(I79,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(J79,$A$6:$A$88,0)),0))</f>
         <v/>
       </c>
       <c r="L79" s="11">
@@ -4943,125 +4959,88 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="7" t="inlineStr">
-        <is>
-          <t>10. בדיקות ומסירה</t>
-        </is>
-      </c>
-      <c r="B80" s="8" t="n"/>
-      <c r="C80" s="8" t="n"/>
-      <c r="D80" s="8" t="n"/>
-      <c r="E80" s="8" t="n"/>
-      <c r="F80" s="8" t="n"/>
-      <c r="G80" s="8" t="n"/>
-      <c r="H80" s="8" t="n"/>
-      <c r="I80" s="8" t="n"/>
-      <c r="J80" s="8" t="n"/>
-      <c r="K80" s="8" t="n"/>
-      <c r="L80" s="8" t="n"/>
-      <c r="M80" s="8" t="n"/>
-      <c r="N80" s="8" t="n"/>
-      <c r="O80" s="8" t="n"/>
-      <c r="P80" s="8" t="n"/>
-      <c r="Q80" s="8" t="n"/>
-      <c r="R80" s="8" t="n"/>
-      <c r="S80" s="8" t="n"/>
-      <c r="T80" s="8" t="n"/>
-      <c r="U80" s="8" t="n"/>
-      <c r="V80" s="8" t="n"/>
-      <c r="W80" s="8" t="n"/>
-      <c r="X80" s="8" t="n"/>
-      <c r="Y80" s="8" t="n"/>
-      <c r="Z80" s="8" t="n"/>
-      <c r="AA80" s="8" t="n"/>
-      <c r="AB80" s="8" t="n"/>
-      <c r="AC80" s="8" t="n"/>
-      <c r="AD80" s="8" t="n"/>
-      <c r="AE80" s="8" t="n"/>
-      <c r="AF80" s="8" t="n"/>
-      <c r="AG80" s="8" t="n"/>
-      <c r="AH80" s="8" t="n"/>
-      <c r="AI80" s="8" t="n"/>
-      <c r="AJ80" s="8" t="n"/>
-      <c r="AK80" s="8" t="n"/>
-      <c r="AL80" s="8" t="n"/>
-      <c r="AM80" s="8" t="n"/>
-      <c r="AN80" s="8" t="n"/>
-      <c r="AO80" s="8" t="n"/>
-      <c r="AP80" s="8" t="n"/>
-      <c r="AQ80" s="8" t="n"/>
-      <c r="AR80" s="8" t="n"/>
-      <c r="AS80" s="8" t="n"/>
-      <c r="AT80" s="8" t="n"/>
-      <c r="AU80" s="8" t="n"/>
-      <c r="AV80" s="8" t="n"/>
-      <c r="AW80" s="8" t="n"/>
-      <c r="AX80" s="8" t="n"/>
-      <c r="AY80" s="8" t="n"/>
-      <c r="AZ80" s="8" t="n"/>
-      <c r="BA80" s="8" t="n"/>
-      <c r="BB80" s="8" t="n"/>
-      <c r="BC80" s="8" t="n"/>
-      <c r="BD80" s="8" t="n"/>
-      <c r="BE80" s="8" t="n"/>
-      <c r="BF80" s="8" t="n"/>
-      <c r="BG80" s="8" t="n"/>
-      <c r="BH80" s="8" t="n"/>
-      <c r="BI80" s="8" t="n"/>
-      <c r="BJ80" s="8" t="n"/>
-      <c r="BK80" s="8" t="n"/>
-      <c r="BL80" s="8" t="n"/>
-      <c r="BM80" s="8" t="n"/>
-      <c r="BN80" s="8" t="n"/>
-      <c r="BO80" s="8" t="n"/>
+      <c r="A80" s="9" t="inlineStr">
+        <is>
+          <t>V010</t>
+        </is>
+      </c>
+      <c r="B80" s="10" t="inlineStr">
+        <is>
+          <t>עבודות עפר ופילוס (65 מ״ר) ומערכת ניקוז מי נגר</t>
+        </is>
+      </c>
+      <c r="C80" s="10" t="inlineStr">
+        <is>
+          <t>17.01, 17.02</t>
+        </is>
+      </c>
+      <c r="D80" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="E80" s="9" t="inlineStr">
+        <is>
+          <t>X020</t>
+        </is>
+      </c>
+      <c r="F80" s="9" t="n"/>
+      <c r="G80" s="9" t="n"/>
+      <c r="H80" s="9" t="n"/>
+      <c r="I80" s="9" t="n"/>
+      <c r="J80" s="9" t="n"/>
+      <c r="K80" s="11">
+        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$88,MATCH(E80,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(F80,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(G80,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(H80,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(I80,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(J80,$A$6:$A$88,0)),0))</f>
+        <v/>
+      </c>
+      <c r="L80" s="11">
+        <f>IF(D80=0,IF(COUNTA(E80:J80)=0,$D$2,K80),WORKDAY.INTL(K80,1,$D$3))</f>
+        <v/>
+      </c>
+      <c r="M80" s="11">
+        <f>IF(D80=0,L80,WORKDAY.INTL(L80,D80-1,$D$3))</f>
+        <v/>
+      </c>
+      <c r="N80" s="9" t="n"/>
+      <c r="O80" s="10" t="inlineStr">
+        <is>
+          <t>הנחה</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="9" t="inlineStr">
         <is>
-          <t>H010</t>
+          <t>V020</t>
         </is>
       </c>
       <c r="B81" s="10" t="inlineStr">
         <is>
-          <t>בדיקת חשמלאי בודק סופית וטופס 4</t>
+          <t>גינון, השקיה, ברזי גינה ותאורת גן</t>
         </is>
       </c>
       <c r="C81" s="10" t="inlineStr">
         <is>
-          <t>06.09</t>
+          <t>17.04, 17.05</t>
         </is>
       </c>
       <c r="D81" s="9" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E81" s="9" t="inlineStr">
         <is>
-          <t>E020</t>
+          <t>V010</t>
         </is>
       </c>
       <c r="F81" s="9" t="inlineStr">
         <is>
-          <t>E030</t>
-        </is>
-      </c>
-      <c r="G81" s="9" t="inlineStr">
-        <is>
-          <t>E040</t>
-        </is>
-      </c>
-      <c r="H81" s="9" t="inlineStr">
-        <is>
-          <t>C020</t>
-        </is>
-      </c>
-      <c r="I81" s="9" t="inlineStr">
-        <is>
-          <t>L030</t>
-        </is>
-      </c>
+          <t>T030</t>
+        </is>
+      </c>
+      <c r="G81" s="9" t="n"/>
+      <c r="H81" s="9" t="n"/>
+      <c r="I81" s="9" t="n"/>
       <c r="J81" s="9" t="n"/>
       <c r="K81" s="11">
-        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$86,MATCH(E81,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(F81,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(G81,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(H81,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(I81,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(J81,$A$6:$A$86,0)),0))</f>
+        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$88,MATCH(E81,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(F81,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(G81,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(H81,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(I81,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(J81,$A$6:$A$88,0)),0))</f>
         <v/>
       </c>
       <c r="L81" s="11">
@@ -5080,75 +5059,92 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="9" t="inlineStr">
-        <is>
-          <t>H020</t>
-        </is>
-      </c>
-      <c r="B82" s="10" t="inlineStr">
-        <is>
-          <t>בדיקות מערכות סופיות: מים, ניקוז, מיזוג</t>
-        </is>
-      </c>
-      <c r="C82" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D82" s="9" t="n">
-        <v>4</v>
-      </c>
-      <c r="E82" s="9" t="inlineStr">
-        <is>
-          <t>P020</t>
-        </is>
-      </c>
-      <c r="F82" s="9" t="inlineStr">
-        <is>
-          <t>M020</t>
-        </is>
-      </c>
-      <c r="G82" s="9" t="n"/>
-      <c r="H82" s="9" t="n"/>
-      <c r="I82" s="9" t="n"/>
-      <c r="J82" s="9" t="n"/>
-      <c r="K82" s="11">
-        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$86,MATCH(E82,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(F82,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(G82,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(H82,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(I82,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(J82,$A$6:$A$86,0)),0))</f>
-        <v/>
-      </c>
-      <c r="L82" s="11">
-        <f>IF(D82=0,IF(COUNTA(E82:J82)=0,$D$2,K82),WORKDAY.INTL(K82,1,$D$3))</f>
-        <v/>
-      </c>
-      <c r="M82" s="11">
-        <f>IF(D82=0,L82,WORKDAY.INTL(L82,D82-1,$D$3))</f>
-        <v/>
-      </c>
-      <c r="N82" s="12" t="inlineStr">
-        <is>
-          <t>כן</t>
-        </is>
-      </c>
-      <c r="O82" s="10" t="inlineStr">
-        <is>
-          <t>הנחה</t>
-        </is>
-      </c>
+      <c r="A82" s="7" t="inlineStr">
+        <is>
+          <t>10. בדיקות ומסירה</t>
+        </is>
+      </c>
+      <c r="B82" s="8" t="n"/>
+      <c r="C82" s="8" t="n"/>
+      <c r="D82" s="8" t="n"/>
+      <c r="E82" s="8" t="n"/>
+      <c r="F82" s="8" t="n"/>
+      <c r="G82" s="8" t="n"/>
+      <c r="H82" s="8" t="n"/>
+      <c r="I82" s="8" t="n"/>
+      <c r="J82" s="8" t="n"/>
+      <c r="K82" s="8" t="n"/>
+      <c r="L82" s="8" t="n"/>
+      <c r="M82" s="8" t="n"/>
+      <c r="N82" s="8" t="n"/>
+      <c r="O82" s="8" t="n"/>
+      <c r="P82" s="8" t="n"/>
+      <c r="Q82" s="8" t="n"/>
+      <c r="R82" s="8" t="n"/>
+      <c r="S82" s="8" t="n"/>
+      <c r="T82" s="8" t="n"/>
+      <c r="U82" s="8" t="n"/>
+      <c r="V82" s="8" t="n"/>
+      <c r="W82" s="8" t="n"/>
+      <c r="X82" s="8" t="n"/>
+      <c r="Y82" s="8" t="n"/>
+      <c r="Z82" s="8" t="n"/>
+      <c r="AA82" s="8" t="n"/>
+      <c r="AB82" s="8" t="n"/>
+      <c r="AC82" s="8" t="n"/>
+      <c r="AD82" s="8" t="n"/>
+      <c r="AE82" s="8" t="n"/>
+      <c r="AF82" s="8" t="n"/>
+      <c r="AG82" s="8" t="n"/>
+      <c r="AH82" s="8" t="n"/>
+      <c r="AI82" s="8" t="n"/>
+      <c r="AJ82" s="8" t="n"/>
+      <c r="AK82" s="8" t="n"/>
+      <c r="AL82" s="8" t="n"/>
+      <c r="AM82" s="8" t="n"/>
+      <c r="AN82" s="8" t="n"/>
+      <c r="AO82" s="8" t="n"/>
+      <c r="AP82" s="8" t="n"/>
+      <c r="AQ82" s="8" t="n"/>
+      <c r="AR82" s="8" t="n"/>
+      <c r="AS82" s="8" t="n"/>
+      <c r="AT82" s="8" t="n"/>
+      <c r="AU82" s="8" t="n"/>
+      <c r="AV82" s="8" t="n"/>
+      <c r="AW82" s="8" t="n"/>
+      <c r="AX82" s="8" t="n"/>
+      <c r="AY82" s="8" t="n"/>
+      <c r="AZ82" s="8" t="n"/>
+      <c r="BA82" s="8" t="n"/>
+      <c r="BB82" s="8" t="n"/>
+      <c r="BC82" s="8" t="n"/>
+      <c r="BD82" s="8" t="n"/>
+      <c r="BE82" s="8" t="n"/>
+      <c r="BF82" s="8" t="n"/>
+      <c r="BG82" s="8" t="n"/>
+      <c r="BH82" s="8" t="n"/>
+      <c r="BI82" s="8" t="n"/>
+      <c r="BJ82" s="8" t="n"/>
+      <c r="BK82" s="8" t="n"/>
+      <c r="BL82" s="8" t="n"/>
+      <c r="BM82" s="8" t="n"/>
+      <c r="BN82" s="8" t="n"/>
+      <c r="BO82" s="8" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="9" t="inlineStr">
         <is>
-          <t>H030</t>
+          <t>H010</t>
         </is>
       </c>
       <c r="B83" s="10" t="inlineStr">
         <is>
-          <t>ניקיון סופי</t>
+          <t>בדיקת חשמלאי בודק סופית וטופס 4</t>
         </is>
       </c>
       <c r="C83" s="10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>06.09</t>
         </is>
       </c>
       <c r="D83" s="9" t="n">
@@ -5156,36 +5152,32 @@
       </c>
       <c r="E83" s="9" t="inlineStr">
         <is>
-          <t>F020</t>
+          <t>E020</t>
         </is>
       </c>
       <c r="F83" s="9" t="inlineStr">
         <is>
-          <t>P020</t>
+          <t>E030</t>
         </is>
       </c>
       <c r="G83" s="9" t="inlineStr">
         <is>
-          <t>V020</t>
+          <t>E040</t>
         </is>
       </c>
       <c r="H83" s="9" t="inlineStr">
         <is>
-          <t>L040</t>
+          <t>C020</t>
         </is>
       </c>
       <c r="I83" s="9" t="inlineStr">
         <is>
-          <t>Z010</t>
-        </is>
-      </c>
-      <c r="J83" s="9" t="inlineStr">
-        <is>
-          <t>L020</t>
-        </is>
-      </c>
+          <t>L030</t>
+        </is>
+      </c>
+      <c r="J83" s="9" t="n"/>
       <c r="K83" s="11">
-        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$86,MATCH(E83,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(F83,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(G83,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(H83,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(I83,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(J83,$A$6:$A$86,0)),0))</f>
+        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$88,MATCH(E83,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(F83,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(G83,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(H83,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(I83,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(J83,$A$6:$A$88,0)),0))</f>
         <v/>
       </c>
       <c r="L83" s="11">
@@ -5206,12 +5198,12 @@
     <row r="84">
       <c r="A84" s="9" t="inlineStr">
         <is>
-          <t>H040</t>
+          <t>H020</t>
         </is>
       </c>
       <c r="B84" s="10" t="inlineStr">
         <is>
-          <t>סיור בדק מול המעצבת ורשימת ליקויים</t>
+          <t>בדיקות מערכות סופיות: מים, ניקוז, מיזוג</t>
         </is>
       </c>
       <c r="C84" s="10" t="inlineStr">
@@ -5220,28 +5212,24 @@
         </is>
       </c>
       <c r="D84" s="9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E84" s="9" t="inlineStr">
         <is>
-          <t>H010</t>
+          <t>P020</t>
         </is>
       </c>
       <c r="F84" s="9" t="inlineStr">
         <is>
-          <t>H020</t>
-        </is>
-      </c>
-      <c r="G84" s="9" t="inlineStr">
-        <is>
-          <t>H030</t>
-        </is>
-      </c>
+          <t>M020</t>
+        </is>
+      </c>
+      <c r="G84" s="9" t="n"/>
       <c r="H84" s="9" t="n"/>
       <c r="I84" s="9" t="n"/>
       <c r="J84" s="9" t="n"/>
       <c r="K84" s="11">
-        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$86,MATCH(E84,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(F84,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(G84,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(H84,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(I84,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(J84,$A$6:$A$86,0)),0))</f>
+        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$88,MATCH(E84,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(F84,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(G84,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(H84,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(I84,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(J84,$A$6:$A$88,0)),0))</f>
         <v/>
       </c>
       <c r="L84" s="11">
@@ -5266,12 +5254,12 @@
     <row r="85">
       <c r="A85" s="9" t="inlineStr">
         <is>
-          <t>H050</t>
+          <t>H030</t>
         </is>
       </c>
       <c r="B85" s="10" t="inlineStr">
         <is>
-          <t>תיקון ליקויים</t>
+          <t>ניקיון סופי</t>
         </is>
       </c>
       <c r="C85" s="10" t="inlineStr">
@@ -5280,20 +5268,40 @@
         </is>
       </c>
       <c r="D85" s="9" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="E85" s="9" t="inlineStr">
         <is>
-          <t>H040</t>
-        </is>
-      </c>
-      <c r="F85" s="9" t="n"/>
-      <c r="G85" s="9" t="n"/>
-      <c r="H85" s="9" t="n"/>
-      <c r="I85" s="9" t="n"/>
-      <c r="J85" s="9" t="n"/>
+          <t>F020</t>
+        </is>
+      </c>
+      <c r="F85" s="9" t="inlineStr">
+        <is>
+          <t>P020</t>
+        </is>
+      </c>
+      <c r="G85" s="9" t="inlineStr">
+        <is>
+          <t>V020</t>
+        </is>
+      </c>
+      <c r="H85" s="9" t="inlineStr">
+        <is>
+          <t>L040</t>
+        </is>
+      </c>
+      <c r="I85" s="9" t="inlineStr">
+        <is>
+          <t>Z010</t>
+        </is>
+      </c>
+      <c r="J85" s="9" t="inlineStr">
+        <is>
+          <t>L020</t>
+        </is>
+      </c>
       <c r="K85" s="11">
-        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$86,MATCH(E85,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(F85,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(G85,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(H85,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(I85,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(J85,$A$6:$A$86,0)),0))</f>
+        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$88,MATCH(E85,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(F85,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(G85,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(H85,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(I85,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(J85,$A$6:$A$88,0)),0))</f>
         <v/>
       </c>
       <c r="L85" s="11">
@@ -5304,11 +5312,7 @@
         <f>IF(D85=0,L85,WORKDAY.INTL(L85,D85-1,$D$3))</f>
         <v/>
       </c>
-      <c r="N85" s="12" t="inlineStr">
-        <is>
-          <t>כן</t>
-        </is>
-      </c>
+      <c r="N85" s="9" t="n"/>
       <c r="O85" s="10" t="inlineStr">
         <is>
           <t>הנחה</t>
@@ -5318,12 +5322,12 @@
     <row r="86">
       <c r="A86" s="9" t="inlineStr">
         <is>
-          <t>H060</t>
+          <t>H040</t>
         </is>
       </c>
       <c r="B86" s="10" t="inlineStr">
         <is>
-          <t>מסירה למזמין</t>
+          <t>סיור בדק מול המעצבת ורשימת ליקויים</t>
         </is>
       </c>
       <c r="C86" s="10" t="inlineStr">
@@ -5332,20 +5336,28 @@
         </is>
       </c>
       <c r="D86" s="9" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E86" s="9" t="inlineStr">
         <is>
-          <t>H050</t>
-        </is>
-      </c>
-      <c r="F86" s="9" t="n"/>
-      <c r="G86" s="9" t="n"/>
+          <t>H010</t>
+        </is>
+      </c>
+      <c r="F86" s="9" t="inlineStr">
+        <is>
+          <t>H020</t>
+        </is>
+      </c>
+      <c r="G86" s="9" t="inlineStr">
+        <is>
+          <t>H030</t>
+        </is>
+      </c>
       <c r="H86" s="9" t="n"/>
       <c r="I86" s="9" t="n"/>
       <c r="J86" s="9" t="n"/>
       <c r="K86" s="11">
-        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$86,MATCH(E86,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(F86,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(G86,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(H86,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(I86,$A$6:$A$86,0)),0),IFERROR(INDEX($M$6:$M$86,MATCH(J86,$A$6:$A$86,0)),0))</f>
+        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$88,MATCH(E86,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(F86,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(G86,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(H86,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(I86,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(J86,$A$6:$A$88,0)),0))</f>
         <v/>
       </c>
       <c r="L86" s="11">
@@ -5363,34 +5375,138 @@
       </c>
       <c r="O86" s="10" t="inlineStr">
         <is>
+          <t>הנחה</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="9" t="inlineStr">
+        <is>
+          <t>H050</t>
+        </is>
+      </c>
+      <c r="B87" s="10" t="inlineStr">
+        <is>
+          <t>תיקון ליקויים</t>
+        </is>
+      </c>
+      <c r="C87" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D87" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="E87" s="9" t="inlineStr">
+        <is>
+          <t>H040</t>
+        </is>
+      </c>
+      <c r="F87" s="9" t="n"/>
+      <c r="G87" s="9" t="n"/>
+      <c r="H87" s="9" t="n"/>
+      <c r="I87" s="9" t="n"/>
+      <c r="J87" s="9" t="n"/>
+      <c r="K87" s="11">
+        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$88,MATCH(E87,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(F87,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(G87,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(H87,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(I87,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(J87,$A$6:$A$88,0)),0))</f>
+        <v/>
+      </c>
+      <c r="L87" s="11">
+        <f>IF(D87=0,IF(COUNTA(E87:J87)=0,$D$2,K87),WORKDAY.INTL(K87,1,$D$3))</f>
+        <v/>
+      </c>
+      <c r="M87" s="11">
+        <f>IF(D87=0,L87,WORKDAY.INTL(L87,D87-1,$D$3))</f>
+        <v/>
+      </c>
+      <c r="N87" s="12" t="inlineStr">
+        <is>
+          <t>כן</t>
+        </is>
+      </c>
+      <c r="O87" s="10" t="inlineStr">
+        <is>
+          <t>הנחה</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="9" t="inlineStr">
+        <is>
+          <t>H060</t>
+        </is>
+      </c>
+      <c r="B88" s="10" t="inlineStr">
+        <is>
+          <t>מסירה למזמין</t>
+        </is>
+      </c>
+      <c r="C88" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D88" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E88" s="9" t="inlineStr">
+        <is>
+          <t>H050</t>
+        </is>
+      </c>
+      <c r="F88" s="9" t="n"/>
+      <c r="G88" s="9" t="n"/>
+      <c r="H88" s="9" t="n"/>
+      <c r="I88" s="9" t="n"/>
+      <c r="J88" s="9" t="n"/>
+      <c r="K88" s="11">
+        <f>MAX($D$2-1,IFERROR(INDEX($M$6:$M$88,MATCH(E88,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(F88,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(G88,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(H88,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(I88,$A$6:$A$88,0)),0),IFERROR(INDEX($M$6:$M$88,MATCH(J88,$A$6:$A$88,0)),0))</f>
+        <v/>
+      </c>
+      <c r="L88" s="11">
+        <f>IF(D88=0,IF(COUNTA(E88:J88)=0,$D$2,K88),WORKDAY.INTL(K88,1,$D$3))</f>
+        <v/>
+      </c>
+      <c r="M88" s="11">
+        <f>IF(D88=0,L88,WORKDAY.INTL(L88,D88-1,$D$3))</f>
+        <v/>
+      </c>
+      <c r="N88" s="12" t="inlineStr">
+        <is>
+          <t>כן</t>
+        </is>
+      </c>
+      <c r="O88" s="10" t="inlineStr">
+        <is>
           <t>אבן דרך</t>
         </is>
       </c>
     </row>
-    <row r="88">
-      <c r="B88" s="13" t="inlineStr">
+    <row r="90">
+      <c r="B90" s="13" t="inlineStr">
         <is>
           <t>סיום הפרויקט (מסירה)</t>
         </is>
       </c>
-      <c r="M88" s="14">
-        <f>MAX($M$6:$M$86)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="89">
-      <c r="B89" s="13" t="inlineStr">
+      <c r="M90" s="14">
+        <f>MAX($M$6:$M$88)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="91">
+      <c r="B91" s="13" t="inlineStr">
         <is>
           <t>משך כולל בשבועות</t>
         </is>
       </c>
-      <c r="M89" s="13">
-        <f>ROUND((M88-$D$2)/7,1)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="90">
-      <c r="B90" t="inlineStr">
+      <c r="M91" s="13">
+        <f>ROUND((M90-$D$2)/7,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="92">
+      <c r="B92" t="inlineStr">
         <is>
           <t>* נתיב קריטי מחושב סטטית בעת יצירת הקובץ לפי המשכים והקודמות שהוגדרו. שינוי משכים לא יעדכן את העמודה.</t>
         </is>
@@ -5400,7 +5516,7 @@
   <mergeCells count="1">
     <mergeCell ref="F2:O3"/>
   </mergeCells>
-  <conditionalFormatting sqref="P6:BO86">
+  <conditionalFormatting sqref="P6:BO88">
     <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="1">
       <formula>AND($D6=0,$A6&lt;&gt;"",$L6&gt;=P$5,$L6&lt;=P$5+6)</formula>
     </cfRule>

</xml_diff>